<commit_message>
update data and cache
</commit_message>
<xml_diff>
--- a/dados/dados_financeiros.xlsx
+++ b/dados/dados_financeiros.xlsx
@@ -1827,11 +1827,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="2007175572"/>
-        <c:axId val="987094786"/>
+        <c:axId val="1003032112"/>
+        <c:axId val="792849031"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2007175572"/>
+        <c:axId val="1003032112"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1883,10 +1883,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="987094786"/>
+        <c:crossAx val="792849031"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="987094786"/>
+        <c:axId val="792849031"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1950,7 +1950,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2007175572"/>
+        <c:crossAx val="1003032112"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -8230,11 +8230,11 @@
       <c r="B18" s="23">
         <v>46145.0</v>
       </c>
-      <c r="C18" s="19">
+      <c r="C18" s="23">
+        <v>46145.0</v>
+      </c>
+      <c r="D18" s="19">
         <v>7600.0</v>
-      </c>
-      <c r="D18" s="9">
-        <v>7000.0</v>
       </c>
       <c r="E18" s="38"/>
     </row>
@@ -10820,7 +10820,7 @@
       </c>
       <c r="K4" s="51">
         <f>SUM(C4:C123)</f>
-        <v>211799.41</v>
+        <v>212399.41</v>
       </c>
       <c r="M4" s="52">
         <v>46054.0</v>
@@ -10860,7 +10860,7 @@
       </c>
       <c r="K5" s="51">
         <f>SUMIFS(D4:D123,A4:A123,"&lt;="&amp;EOMONTH(TODAY(),0)+1-1,A4:A123,"&lt;&gt;")</f>
-        <v>14883.12</v>
+        <v>17529.01</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="1">
@@ -10897,7 +10897,7 @@
       </c>
       <c r="K6" s="51">
         <f>G17</f>
-        <v>981.56</v>
+        <v>1581.56</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="1">
@@ -10911,11 +10911,11 @@
       </c>
       <c r="C7" s="56">
         <f>IF($A7="","",SUMIFS('Inventário de Lotes'!$D:$D,'Inventário de Lotes'!$B:$B,"&gt;="&amp;$A7,'Inventário de Lotes'!$B:$B,"&lt;"&amp;EDATE($A7,1)))</f>
-        <v>16280</v>
+        <v>16880</v>
       </c>
       <c r="D7" s="56">
         <f t="shared" si="1"/>
-        <v>2045.89</v>
+        <v>2645.89</v>
       </c>
       <c r="E7" s="57">
         <f>IF($A7="","",COUNTIFS('Todos os Gastos'!$A:$A,"&gt;="&amp;$A7,'Todos os Gastos'!$A:$A,"&lt;"&amp;EDATE($A7,1)))</f>
@@ -10927,14 +10927,14 @@
       </c>
       <c r="G7" s="56">
         <f t="shared" si="2"/>
-        <v>16929.01</v>
+        <v>17529.01</v>
       </c>
       <c r="J7" s="50" t="s">
         <v>119</v>
       </c>
       <c r="K7" s="51">
         <f>SUMIFS(D4:D123,A4:A123,"&gt;="&amp;EOMONTH(TODAY(),-1)+1,A4:A123,"&lt;"&amp;EDATE(EOMONTH(TODAY(),-1)+1,1))</f>
-        <v>-2631.35</v>
+        <v>2645.89</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
@@ -10964,14 +10964,14 @@
       </c>
       <c r="G8" s="53">
         <f t="shared" si="2"/>
-        <v>17564.83</v>
+        <v>18164.83</v>
       </c>
       <c r="J8" s="50" t="s">
         <v>120</v>
       </c>
       <c r="K8" s="51">
         <f>AVERAGEIF(D4:D123,"&lt;&gt;",D4:D123)</f>
-        <v>70.11142857</v>
+        <v>112.9685714</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="1">
@@ -11001,7 +11001,7 @@
       </c>
       <c r="G9" s="56">
         <f t="shared" si="2"/>
-        <v>16980.65</v>
+        <v>17580.65</v>
       </c>
       <c r="J9" s="50" t="s">
         <v>121</v>
@@ -11038,7 +11038,7 @@
       </c>
       <c r="G10" s="53">
         <f t="shared" si="2"/>
-        <v>15836.47</v>
+        <v>16436.47</v>
       </c>
       <c r="J10" s="50" t="s">
         <v>122</v>
@@ -11075,7 +11075,7 @@
       </c>
       <c r="G11" s="56">
         <f t="shared" si="2"/>
-        <v>14042.29</v>
+        <v>14642.29</v>
       </c>
       <c r="J11" s="50" t="s">
         <v>123</v>
@@ -11112,14 +11112,14 @@
       </c>
       <c r="G12" s="53">
         <f t="shared" si="2"/>
-        <v>12648.31</v>
+        <v>13248.31</v>
       </c>
       <c r="J12" s="50" t="s">
         <v>124</v>
       </c>
       <c r="K12" s="58" t="str">
         <f>TEXT(TODAY(),"mmm/yy")</f>
-        <v>abr./26</v>
+        <v>mai./26</v>
       </c>
     </row>
     <row r="13" ht="15.0" customHeight="1">
@@ -11149,7 +11149,7 @@
       </c>
       <c r="G13" s="56">
         <f t="shared" si="2"/>
-        <v>11754.13</v>
+        <v>12354.13</v>
       </c>
     </row>
     <row r="14" ht="15.0" customHeight="1">
@@ -11179,7 +11179,7 @@
       </c>
       <c r="G14" s="53">
         <f t="shared" si="2"/>
-        <v>7339.95</v>
+        <v>7939.95</v>
       </c>
       <c r="J14" s="59"/>
     </row>
@@ -11210,7 +11210,7 @@
       </c>
       <c r="G15" s="56">
         <f t="shared" si="2"/>
-        <v>7431.1</v>
+        <v>8031.1</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1">
@@ -11240,7 +11240,7 @@
       </c>
       <c r="G16" s="53">
         <f t="shared" si="2"/>
-        <v>4375.15</v>
+        <v>4975.15</v>
       </c>
     </row>
     <row r="17" ht="15.0" customHeight="1">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="G17" s="56">
         <f t="shared" si="2"/>
-        <v>981.56</v>
+        <v>1581.56</v>
       </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">

</xml_diff>

<commit_message>
update data e cache
</commit_message>
<xml_diff>
--- a/dados/dados_financeiros.xlsx
+++ b/dados/dados_financeiros.xlsx
@@ -9,7 +9,7 @@
     <sheet state="visible" name="Carteira" sheetId="4" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Todos os Gastos'!$A$1:$E$225</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Todos os Gastos'!$A$1:$E$226</definedName>
     <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Inventário de Lotes'!$A$1:$E$45</definedName>
     <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'Resumo Mensal'!$A$3:$G$123</definedName>
     <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">Carteira!$A$1:$AY$85</definedName>
@@ -20,14 +20,14 @@
   </pivotCaches>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="pJRHvcXxvrt2iyftP589alz4iTYJ/TjvnqN2pkLwSTU="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="YykOvY0Bmv9mpsg5RxHSAPHLZ3zOFxgZyJrEMKXXMP4="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2228" uniqueCount="444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2229" uniqueCount="444">
   <si>
     <t>Data</t>
   </si>
@@ -1909,11 +1909,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1169612973"/>
-        <c:axId val="1320945558"/>
+        <c:axId val="1232310031"/>
+        <c:axId val="1471548968"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1169612973"/>
+        <c:axId val="1232310031"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1965,10 +1965,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1320945558"/>
+        <c:crossAx val="1471548968"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1320945558"/>
+        <c:axId val="1471548968"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2032,7 +2032,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1169612973"/>
+        <c:crossAx val="1232310031"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2171,7 +2171,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" invalid="1" refreshOnLoad="1">
   <cacheSource type="worksheet">
-    <worksheetSource ref="C1:E1014" sheet="Todos os Gastos"/>
+    <worksheetSource ref="C1:E1015" sheet="Todos os Gastos"/>
   </cacheSource>
   <cacheFields>
     <cacheField name="Valor" numFmtId="2">
@@ -4340,8 +4340,8 @@
       <c r="H80" s="28"/>
     </row>
     <row r="81" ht="14.25" customHeight="1">
-      <c r="A81" s="23">
-        <v>46150.0</v>
+      <c r="A81" s="25">
+        <v>46149.0</v>
       </c>
       <c r="B81" s="8" t="s">
         <v>52</v>
@@ -4353,40 +4353,40 @@
       <c r="H81" s="28"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
-      <c r="A82" s="23">
-        <v>46150.0</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C82" s="9">
-        <v>65.0</v>
+      <c r="A82" s="25">
+        <v>46149.0</v>
+      </c>
+      <c r="B82" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="C82" s="19">
+        <v>120.0</v>
       </c>
       <c r="G82" s="9"/>
       <c r="H82" s="28"/>
     </row>
     <row r="83" ht="14.25" customHeight="1">
       <c r="A83" s="23">
-        <v>46153.0</v>
-      </c>
-      <c r="B83" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C83" s="19">
-        <v>98.88</v>
+        <v>46150.0</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C83" s="9">
+        <v>65.0</v>
       </c>
       <c r="G83" s="9"/>
       <c r="H83" s="28"/>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="23">
-        <v>46154.0</v>
+        <v>46153.0</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="C84" s="19">
-        <v>980.86</v>
+        <v>98.88</v>
       </c>
       <c r="G84" s="9"/>
       <c r="H84" s="28"/>
@@ -4396,10 +4396,10 @@
         <v>46154.0</v>
       </c>
       <c r="B85" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C85" s="3">
-        <v>2831.4</v>
+        <v>25</v>
+      </c>
+      <c r="C85" s="19">
+        <v>980.86</v>
       </c>
       <c r="G85" s="9"/>
       <c r="H85" s="28"/>
@@ -4409,36 +4409,36 @@
         <v>46154.0</v>
       </c>
       <c r="B86" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C86" s="9">
-        <v>50.0</v>
+        <v>33</v>
+      </c>
+      <c r="C86" s="3">
+        <v>2831.4</v>
       </c>
       <c r="G86" s="9"/>
       <c r="H86" s="28"/>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="23">
-        <v>46157.0</v>
+        <v>46154.0</v>
       </c>
       <c r="B87" s="8" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="C87" s="9">
-        <v>132.4</v>
+        <v>50.0</v>
       </c>
       <c r="G87" s="9"/>
       <c r="H87" s="28"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="23">
-        <v>46162.0</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C88" s="19">
-        <v>5372.0</v>
+        <v>46157.0</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C88" s="9">
+        <v>132.4</v>
       </c>
       <c r="G88" s="9"/>
       <c r="H88" s="28"/>
@@ -4447,37 +4447,37 @@
       <c r="A89" s="23">
         <v>46162.0</v>
       </c>
-      <c r="B89" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C89" s="9">
-        <v>113.31</v>
+      <c r="B89" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C89" s="19">
+        <v>5372.0</v>
       </c>
       <c r="G89" s="9"/>
       <c r="H89" s="28"/>
     </row>
     <row r="90" ht="14.25" customHeight="1">
-      <c r="A90" s="1">
-        <v>46175.0</v>
+      <c r="A90" s="23">
+        <v>46162.0</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C90" s="9">
-        <v>580.0</v>
+        <v>113.31</v>
       </c>
       <c r="G90" s="9"/>
       <c r="H90" s="28"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
-      <c r="A91" s="23">
-        <v>46178.0</v>
+      <c r="A91" s="1">
+        <v>46175.0</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C91" s="9">
-        <v>195.0</v>
+        <v>580.0</v>
       </c>
       <c r="G91" s="9"/>
       <c r="H91" s="28"/>
@@ -4487,36 +4487,36 @@
         <v>46178.0</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C92" s="9">
-        <v>950.0</v>
+        <v>195.0</v>
       </c>
       <c r="G92" s="9"/>
       <c r="H92" s="28"/>
     </row>
     <row r="93" ht="14.25" customHeight="1">
-      <c r="A93" s="1">
-        <v>46181.0</v>
+      <c r="A93" s="23">
+        <v>46178.0</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C93" s="9">
-        <v>120.0</v>
+        <v>950.0</v>
       </c>
       <c r="G93" s="9"/>
       <c r="H93" s="28"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="1">
-        <v>46183.0</v>
-      </c>
-      <c r="B94" s="2" t="s">
-        <v>38</v>
+        <v>46181.0</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="C94" s="9">
-        <v>65.0</v>
+        <v>120.0</v>
       </c>
       <c r="G94" s="9"/>
       <c r="H94" s="28"/>
@@ -4525,11 +4525,11 @@
       <c r="A95" s="1">
         <v>46183.0</v>
       </c>
-      <c r="B95" s="8" t="s">
-        <v>44</v>
+      <c r="B95" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C95" s="9">
-        <v>50.0</v>
+        <v>65.0</v>
       </c>
       <c r="G95" s="9"/>
       <c r="H95" s="28"/>
@@ -4539,36 +4539,36 @@
         <v>46183.0</v>
       </c>
       <c r="B96" s="8" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="C96" s="9">
-        <v>530.0</v>
+        <v>50.0</v>
       </c>
       <c r="G96" s="9"/>
       <c r="H96" s="28"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="1">
-        <v>46184.0</v>
+        <v>46183.0</v>
       </c>
       <c r="B97" s="8" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="C97" s="9">
-        <v>95.12</v>
+        <v>530.0</v>
       </c>
       <c r="G97" s="9"/>
       <c r="H97" s="28"/>
     </row>
     <row r="98" ht="14.25" customHeight="1">
-      <c r="A98" s="23">
-        <v>46185.0</v>
+      <c r="A98" s="1">
+        <v>46184.0</v>
       </c>
       <c r="B98" s="8" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="C98" s="9">
-        <v>981.95</v>
+        <v>95.12</v>
       </c>
       <c r="G98" s="9"/>
       <c r="H98" s="28"/>
@@ -4578,36 +4578,36 @@
         <v>46185.0</v>
       </c>
       <c r="B99" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C99" s="3">
-        <v>2831.4</v>
+        <v>25</v>
+      </c>
+      <c r="C99" s="9">
+        <v>981.95</v>
       </c>
       <c r="G99" s="9"/>
       <c r="H99" s="28"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="23">
-        <v>46188.0</v>
+        <v>46185.0</v>
       </c>
       <c r="B100" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C100" s="9">
-        <v>132.4</v>
+        <v>33</v>
+      </c>
+      <c r="C100" s="3">
+        <v>2831.4</v>
       </c>
       <c r="G100" s="9"/>
       <c r="H100" s="28"/>
     </row>
     <row r="101" ht="14.25" customHeight="1">
       <c r="A101" s="23">
-        <v>46192.0</v>
-      </c>
-      <c r="B101" s="2" t="s">
-        <v>23</v>
+        <v>46188.0</v>
+      </c>
+      <c r="B101" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="C101" s="9">
-        <v>7200.0</v>
+        <v>132.4</v>
       </c>
       <c r="G101" s="9"/>
       <c r="H101" s="28"/>
@@ -4616,37 +4616,37 @@
       <c r="A102" s="23">
         <v>46192.0</v>
       </c>
-      <c r="B102" s="8" t="s">
-        <v>40</v>
+      <c r="B102" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C102" s="9">
-        <v>113.31</v>
+        <v>7200.0</v>
       </c>
       <c r="G102" s="9"/>
       <c r="H102" s="28"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
-      <c r="A103" s="1">
-        <v>46205.0</v>
+      <c r="A103" s="23">
+        <v>46192.0</v>
       </c>
       <c r="B103" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C103" s="9">
-        <v>930.0</v>
+        <v>113.31</v>
       </c>
       <c r="G103" s="9"/>
       <c r="H103" s="28"/>
     </row>
     <row r="104" ht="14.25" customHeight="1">
-      <c r="A104" s="23">
-        <v>46209.0</v>
+      <c r="A104" s="1">
+        <v>46205.0</v>
       </c>
       <c r="B104" s="8" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C104" s="9">
-        <v>195.0</v>
+        <v>930.0</v>
       </c>
       <c r="G104" s="9"/>
       <c r="H104" s="28"/>
@@ -4656,49 +4656,49 @@
         <v>46209.0</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C105" s="9">
-        <v>950.0</v>
+        <v>195.0</v>
       </c>
       <c r="G105" s="9"/>
       <c r="H105" s="28"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="23">
-        <v>46211.0</v>
+        <v>46209.0</v>
       </c>
       <c r="B106" s="8" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C106" s="9">
-        <v>120.0</v>
+        <v>950.0</v>
       </c>
       <c r="G106" s="9"/>
       <c r="H106" s="28"/>
     </row>
     <row r="107" ht="14.25" customHeight="1">
-      <c r="A107" s="1">
-        <v>46213.0</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>38</v>
+      <c r="A107" s="23">
+        <v>46211.0</v>
+      </c>
+      <c r="B107" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="C107" s="9">
-        <v>65.0</v>
+        <v>120.0</v>
       </c>
       <c r="G107" s="9"/>
       <c r="H107" s="28"/>
     </row>
     <row r="108" ht="14.25" customHeight="1">
-      <c r="A108" s="23">
-        <v>46216.0</v>
-      </c>
-      <c r="B108" s="8" t="s">
-        <v>25</v>
+      <c r="A108" s="1">
+        <v>46213.0</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C108" s="9">
-        <v>981.95</v>
+        <v>65.0</v>
       </c>
       <c r="G108" s="9"/>
       <c r="H108" s="28"/>
@@ -4708,10 +4708,10 @@
         <v>46216.0</v>
       </c>
       <c r="B109" s="8" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="C109" s="9">
-        <v>95.12</v>
+        <v>981.95</v>
       </c>
       <c r="G109" s="9"/>
       <c r="H109" s="28"/>
@@ -4721,23 +4721,23 @@
         <v>46216.0</v>
       </c>
       <c r="B110" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C110" s="3">
-        <v>2831.4</v>
+        <v>43</v>
+      </c>
+      <c r="C110" s="9">
+        <v>95.12</v>
       </c>
       <c r="G110" s="9"/>
       <c r="H110" s="28"/>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="23">
-        <v>46218.0</v>
+        <v>46216.0</v>
       </c>
       <c r="B111" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C111" s="9">
-        <v>132.4</v>
+        <v>33</v>
+      </c>
+      <c r="C111" s="3">
+        <v>2831.4</v>
       </c>
       <c r="G111" s="9"/>
       <c r="H111" s="28"/>
@@ -4747,23 +4747,23 @@
         <v>46218.0</v>
       </c>
       <c r="B112" s="8" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="C112" s="9">
-        <v>50.0</v>
+        <v>132.4</v>
       </c>
       <c r="G112" s="9"/>
       <c r="H112" s="28"/>
     </row>
     <row r="113" ht="14.25" customHeight="1">
       <c r="A113" s="23">
-        <v>46223.0</v>
-      </c>
-      <c r="B113" s="2" t="s">
-        <v>23</v>
+        <v>46218.0</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>44</v>
       </c>
       <c r="C113" s="9">
-        <v>6800.0</v>
+        <v>50.0</v>
       </c>
       <c r="G113" s="9"/>
       <c r="H113" s="28"/>
@@ -4772,53 +4772,50 @@
       <c r="A114" s="23">
         <v>46223.0</v>
       </c>
-      <c r="B114" s="8" t="s">
-        <v>40</v>
+      <c r="B114" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C114" s="9">
-        <v>113.31</v>
+        <v>6800.0</v>
       </c>
       <c r="G114" s="9"/>
       <c r="H114" s="28"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
-      <c r="A115" s="1">
-        <v>46237.0</v>
+      <c r="A115" s="23">
+        <v>46223.0</v>
       </c>
       <c r="B115" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C115" s="9">
-        <v>1500.0</v>
+        <v>113.31</v>
       </c>
       <c r="G115" s="9"/>
       <c r="H115" s="28"/>
     </row>
     <row r="116" ht="14.25" customHeight="1">
-      <c r="A116" s="23">
-        <v>46239.0</v>
+      <c r="A116" s="1">
+        <v>46237.0</v>
       </c>
       <c r="B116" s="8" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="C116" s="9">
-        <v>950.0</v>
-      </c>
-      <c r="F116" s="26"/>
-      <c r="G116" s="12"/>
-      <c r="H116" s="21"/>
-      <c r="I116" s="14"/>
-      <c r="J116" s="14"/>
+        <v>1500.0</v>
+      </c>
+      <c r="G116" s="9"/>
+      <c r="H116" s="28"/>
     </row>
     <row r="117" ht="14.25" customHeight="1">
       <c r="A117" s="23">
-        <v>46240.0</v>
+        <v>46239.0</v>
       </c>
       <c r="B117" s="8" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C117" s="9">
-        <v>195.0</v>
+        <v>950.0</v>
       </c>
       <c r="F117" s="26"/>
       <c r="G117" s="12"/>
@@ -4831,49 +4828,52 @@
         <v>46240.0</v>
       </c>
       <c r="B118" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C118" s="9">
+        <v>195.0</v>
+      </c>
+      <c r="F118" s="26"/>
+      <c r="G118" s="12"/>
+      <c r="H118" s="21"/>
+      <c r="I118" s="14"/>
+      <c r="J118" s="14"/>
+    </row>
+    <row r="119" ht="14.25" customHeight="1">
+      <c r="A119" s="23">
+        <v>46240.0</v>
+      </c>
+      <c r="B119" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C118" s="9">
+      <c r="C119" s="9">
         <v>120.0</v>
-      </c>
-      <c r="G118" s="9"/>
-      <c r="H118" s="28"/>
-    </row>
-    <row r="119" ht="14.25" customHeight="1">
-      <c r="A119" s="1">
-        <v>46244.0</v>
-      </c>
-      <c r="B119" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C119" s="9">
-        <v>65.0</v>
       </c>
       <c r="G119" s="9"/>
       <c r="H119" s="28"/>
     </row>
     <row r="120" ht="14.25" customHeight="1">
-      <c r="A120" s="23">
-        <v>46245.0</v>
-      </c>
-      <c r="B120" s="8" t="s">
-        <v>43</v>
+      <c r="A120" s="1">
+        <v>46244.0</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C120" s="9">
-        <v>95.12</v>
+        <v>65.0</v>
       </c>
       <c r="G120" s="9"/>
       <c r="H120" s="28"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
-      <c r="A121" s="1">
-        <v>46246.0</v>
+      <c r="A121" s="23">
+        <v>46245.0</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="C121" s="9">
-        <v>981.95</v>
+        <v>95.12</v>
       </c>
       <c r="G121" s="9"/>
       <c r="H121" s="28"/>
@@ -4883,10 +4883,10 @@
         <v>46246.0</v>
       </c>
       <c r="B122" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C122" s="3">
-        <v>2831.4</v>
+        <v>25</v>
+      </c>
+      <c r="C122" s="9">
+        <v>981.95</v>
       </c>
       <c r="G122" s="9"/>
       <c r="H122" s="28"/>
@@ -4896,10 +4896,10 @@
         <v>46246.0</v>
       </c>
       <c r="B123" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C123" s="9">
-        <v>460.0</v>
+        <v>33</v>
+      </c>
+      <c r="C123" s="3">
+        <v>2831.4</v>
       </c>
       <c r="G123" s="9"/>
       <c r="H123" s="28"/>
@@ -4909,10 +4909,10 @@
         <v>46246.0</v>
       </c>
       <c r="B124" s="8" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C124" s="9">
-        <v>50.0</v>
+        <v>460.0</v>
       </c>
       <c r="G124" s="9"/>
       <c r="H124" s="28"/>
@@ -4922,36 +4922,36 @@
         <v>46246.0</v>
       </c>
       <c r="B125" s="8" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="C125" s="9">
-        <v>530.0</v>
+        <v>50.0</v>
       </c>
       <c r="G125" s="9"/>
       <c r="H125" s="28"/>
     </row>
     <row r="126" ht="14.25" customHeight="1">
-      <c r="A126" s="23">
-        <v>46249.0</v>
+      <c r="A126" s="1">
+        <v>46246.0</v>
       </c>
       <c r="B126" s="8" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="C126" s="9">
-        <v>132.4</v>
+        <v>530.0</v>
       </c>
       <c r="G126" s="9"/>
       <c r="H126" s="28"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="A127" s="23">
-        <v>46254.0</v>
-      </c>
-      <c r="B127" s="2" t="s">
-        <v>23</v>
+        <v>46249.0</v>
+      </c>
+      <c r="B127" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="C127" s="9">
-        <v>5800.0</v>
+        <v>132.4</v>
       </c>
       <c r="G127" s="9"/>
       <c r="H127" s="28"/>
@@ -4960,63 +4960,63 @@
       <c r="A128" s="23">
         <v>46254.0</v>
       </c>
-      <c r="B128" s="8" t="s">
-        <v>40</v>
+      <c r="B128" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C128" s="9">
-        <v>113.31</v>
+        <v>5800.0</v>
       </c>
       <c r="G128" s="9"/>
       <c r="H128" s="28"/>
     </row>
     <row r="129" ht="14.25" customHeight="1">
-      <c r="A129" s="1">
-        <v>46267.0</v>
+      <c r="A129" s="23">
+        <v>46254.0</v>
       </c>
       <c r="B129" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C129" s="9">
-        <v>2000.0</v>
+        <v>113.31</v>
       </c>
       <c r="G129" s="9"/>
       <c r="H129" s="28"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
-      <c r="A130" s="23">
-        <v>46269.0</v>
+      <c r="A130" s="1">
+        <v>46267.0</v>
       </c>
       <c r="B130" s="8" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="C130" s="9">
-        <v>950.0</v>
+        <v>2000.0</v>
       </c>
       <c r="G130" s="9"/>
       <c r="H130" s="28"/>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="A131" s="23">
-        <v>46271.0</v>
+        <v>46269.0</v>
       </c>
       <c r="B131" s="8" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C131" s="9">
-        <v>195.0</v>
+        <v>950.0</v>
       </c>
       <c r="G131" s="9"/>
       <c r="H131" s="28"/>
     </row>
     <row r="132" ht="14.25" customHeight="1">
       <c r="A132" s="23">
-        <v>46273.0</v>
+        <v>46271.0</v>
       </c>
       <c r="B132" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C132" s="9">
-        <v>120.0</v>
+        <v>195.0</v>
       </c>
       <c r="G132" s="9"/>
       <c r="H132" s="28"/>
@@ -5026,49 +5026,49 @@
         <v>46273.0</v>
       </c>
       <c r="B133" s="8" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="C133" s="9">
-        <v>90.0</v>
+        <v>120.0</v>
       </c>
       <c r="G133" s="9"/>
       <c r="H133" s="28"/>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="A134" s="23">
-        <v>46274.0</v>
+        <v>46273.0</v>
       </c>
       <c r="B134" s="8" t="s">
-        <v>44</v>
+        <v>73</v>
       </c>
       <c r="C134" s="9">
-        <v>50.0</v>
+        <v>90.0</v>
       </c>
       <c r="G134" s="9"/>
       <c r="H134" s="28"/>
     </row>
     <row r="135" ht="14.25" customHeight="1">
-      <c r="A135" s="1">
-        <v>46275.0</v>
-      </c>
-      <c r="B135" s="2" t="s">
-        <v>38</v>
+      <c r="A135" s="23">
+        <v>46274.0</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>44</v>
       </c>
       <c r="C135" s="9">
-        <v>65.0</v>
+        <v>50.0</v>
       </c>
       <c r="G135" s="9"/>
       <c r="H135" s="28"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
-      <c r="A136" s="23">
-        <v>46276.0</v>
-      </c>
-      <c r="B136" s="8" t="s">
-        <v>25</v>
+      <c r="A136" s="1">
+        <v>46275.0</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C136" s="9">
-        <v>981.95</v>
+        <v>65.0</v>
       </c>
       <c r="G136" s="9"/>
       <c r="H136" s="28"/>
@@ -5078,10 +5078,10 @@
         <v>46276.0</v>
       </c>
       <c r="B137" s="8" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="C137" s="9">
-        <v>95.12</v>
+        <v>981.95</v>
       </c>
       <c r="G137" s="9"/>
       <c r="H137" s="28"/>
@@ -5091,114 +5091,114 @@
         <v>46276.0</v>
       </c>
       <c r="B138" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C138" s="3">
-        <v>2831.4</v>
+        <v>43</v>
+      </c>
+      <c r="C138" s="9">
+        <v>95.12</v>
       </c>
       <c r="G138" s="9"/>
       <c r="H138" s="28"/>
     </row>
     <row r="139" ht="14.25" customHeight="1">
       <c r="A139" s="23">
-        <v>46280.0</v>
+        <v>46276.0</v>
       </c>
       <c r="B139" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C139" s="9">
-        <v>132.4</v>
+        <v>33</v>
+      </c>
+      <c r="C139" s="3">
+        <v>2831.4</v>
       </c>
       <c r="G139" s="9"/>
       <c r="H139" s="28"/>
     </row>
     <row r="140" ht="14.25" customHeight="1">
       <c r="A140" s="23">
-        <v>46285.0</v>
-      </c>
-      <c r="B140" s="2" t="s">
-        <v>23</v>
+        <v>46280.0</v>
+      </c>
+      <c r="B140" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="C140" s="9">
-        <v>6850.0</v>
+        <v>132.4</v>
       </c>
       <c r="G140" s="9"/>
       <c r="H140" s="28"/>
     </row>
     <row r="141" ht="14.25" customHeight="1">
       <c r="A141" s="23">
-        <v>46286.0</v>
-      </c>
-      <c r="B141" s="8" t="s">
-        <v>40</v>
+        <v>46285.0</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C141" s="9">
-        <v>113.31</v>
+        <v>6850.0</v>
       </c>
       <c r="G141" s="9"/>
       <c r="H141" s="28"/>
     </row>
     <row r="142" ht="14.25" customHeight="1">
-      <c r="A142" s="1">
-        <v>46297.0</v>
+      <c r="A142" s="23">
+        <v>46286.0</v>
       </c>
       <c r="B142" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C142" s="9">
-        <v>1800.0</v>
+        <v>113.31</v>
       </c>
       <c r="G142" s="9"/>
       <c r="H142" s="28"/>
     </row>
     <row r="143" ht="14.25" customHeight="1">
-      <c r="A143" s="23">
-        <v>46300.0</v>
+      <c r="A143" s="1">
+        <v>46297.0</v>
       </c>
       <c r="B143" s="8" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="C143" s="9">
-        <v>950.0</v>
+        <v>1800.0</v>
       </c>
       <c r="G143" s="9"/>
       <c r="H143" s="28"/>
     </row>
     <row r="144" ht="14.25" customHeight="1">
       <c r="A144" s="23">
-        <v>46301.0</v>
+        <v>46300.0</v>
       </c>
       <c r="B144" s="8" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C144" s="9">
-        <v>195.0</v>
+        <v>950.0</v>
       </c>
       <c r="G144" s="9"/>
       <c r="H144" s="28"/>
     </row>
     <row r="145" ht="14.25" customHeight="1">
-      <c r="A145" s="1">
-        <v>46302.0</v>
+      <c r="A145" s="23">
+        <v>46301.0</v>
       </c>
       <c r="B145" s="8" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="C145" s="9">
-        <v>530.0</v>
+        <v>195.0</v>
       </c>
       <c r="G145" s="9"/>
       <c r="H145" s="28"/>
     </row>
     <row r="146" ht="14.25" customHeight="1">
       <c r="A146" s="1">
-        <v>46303.0</v>
+        <v>46302.0</v>
       </c>
       <c r="B146" s="8" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C146" s="9">
-        <v>120.0</v>
+        <v>530.0</v>
       </c>
       <c r="G146" s="9"/>
       <c r="H146" s="28"/>
@@ -5208,10 +5208,10 @@
         <v>46303.0</v>
       </c>
       <c r="B147" s="8" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="C147" s="9">
-        <v>90.0</v>
+        <v>120.0</v>
       </c>
       <c r="G147" s="9"/>
       <c r="H147" s="28"/>
@@ -5221,36 +5221,36 @@
         <v>46303.0</v>
       </c>
       <c r="B148" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C148" s="9">
-        <v>119.8</v>
+        <v>90.0</v>
       </c>
       <c r="G148" s="9"/>
       <c r="H148" s="28"/>
     </row>
     <row r="149" ht="14.25" customHeight="1">
       <c r="A149" s="1">
-        <v>46305.0</v>
-      </c>
-      <c r="B149" s="2" t="s">
-        <v>38</v>
+        <v>46303.0</v>
+      </c>
+      <c r="B149" s="8" t="s">
+        <v>74</v>
       </c>
       <c r="C149" s="9">
-        <v>65.0</v>
+        <v>119.8</v>
       </c>
       <c r="G149" s="9"/>
       <c r="H149" s="28"/>
     </row>
     <row r="150" ht="14.25" customHeight="1">
-      <c r="A150" s="23">
-        <v>46308.0</v>
-      </c>
-      <c r="B150" s="8" t="s">
-        <v>25</v>
+      <c r="A150" s="1">
+        <v>46305.0</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C150" s="9">
-        <v>981.95</v>
+        <v>65.0</v>
       </c>
       <c r="G150" s="9"/>
       <c r="H150" s="28"/>
@@ -5260,10 +5260,10 @@
         <v>46308.0</v>
       </c>
       <c r="B151" s="8" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="C151" s="9">
-        <v>95.12</v>
+        <v>981.95</v>
       </c>
       <c r="G151" s="9"/>
       <c r="H151" s="28"/>
@@ -5273,10 +5273,10 @@
         <v>46308.0</v>
       </c>
       <c r="B152" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C152" s="3">
-        <v>2831.4</v>
+        <v>43</v>
+      </c>
+      <c r="C152" s="9">
+        <v>95.12</v>
       </c>
       <c r="G152" s="9"/>
       <c r="H152" s="28"/>
@@ -5286,36 +5286,36 @@
         <v>46308.0</v>
       </c>
       <c r="B153" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C153" s="9">
-        <v>50.0</v>
+        <v>33</v>
+      </c>
+      <c r="C153" s="3">
+        <v>2831.4</v>
       </c>
       <c r="G153" s="9"/>
       <c r="H153" s="28"/>
     </row>
     <row r="154" ht="14.25" customHeight="1">
       <c r="A154" s="23">
-        <v>46310.0</v>
+        <v>46308.0</v>
       </c>
       <c r="B154" s="8" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="C154" s="9">
-        <v>132.4</v>
+        <v>50.0</v>
       </c>
       <c r="G154" s="9"/>
       <c r="H154" s="28"/>
     </row>
     <row r="155" ht="14.25" customHeight="1">
-      <c r="A155" s="1">
-        <v>46315.0</v>
-      </c>
-      <c r="B155" s="2" t="s">
-        <v>23</v>
+      <c r="A155" s="23">
+        <v>46310.0</v>
+      </c>
+      <c r="B155" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="C155" s="9">
-        <v>6000.0</v>
+        <v>132.4</v>
       </c>
       <c r="G155" s="9"/>
       <c r="H155" s="28"/>
@@ -5324,37 +5324,37 @@
       <c r="A156" s="1">
         <v>46315.0</v>
       </c>
-      <c r="B156" s="8" t="s">
-        <v>40</v>
+      <c r="B156" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C156" s="9">
-        <v>113.31</v>
+        <v>6000.0</v>
       </c>
       <c r="G156" s="9"/>
       <c r="H156" s="28"/>
     </row>
     <row r="157" ht="14.25" customHeight="1">
       <c r="A157" s="1">
-        <v>46329.0</v>
+        <v>46315.0</v>
       </c>
       <c r="B157" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C157" s="9">
-        <v>2200.0</v>
+        <v>113.31</v>
       </c>
       <c r="G157" s="9"/>
       <c r="H157" s="28"/>
     </row>
     <row r="158" ht="14.25" customHeight="1">
-      <c r="A158" s="23">
-        <v>46332.0</v>
+      <c r="A158" s="1">
+        <v>46329.0</v>
       </c>
       <c r="B158" s="8" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C158" s="9">
-        <v>195.0</v>
+        <v>2200.0</v>
       </c>
       <c r="G158" s="9"/>
       <c r="H158" s="28"/>
@@ -5364,23 +5364,23 @@
         <v>46332.0</v>
       </c>
       <c r="B159" s="8" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C159" s="9">
-        <v>950.0</v>
+        <v>195.0</v>
       </c>
       <c r="G159" s="9"/>
       <c r="H159" s="28"/>
     </row>
     <row r="160" ht="14.25" customHeight="1">
       <c r="A160" s="23">
-        <v>46335.0</v>
+        <v>46332.0</v>
       </c>
       <c r="B160" s="8" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C160" s="9">
-        <v>120.0</v>
+        <v>950.0</v>
       </c>
       <c r="G160" s="9"/>
       <c r="H160" s="28"/>
@@ -5390,36 +5390,36 @@
         <v>46335.0</v>
       </c>
       <c r="B161" s="8" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="C161" s="9">
-        <v>90.0</v>
+        <v>120.0</v>
       </c>
       <c r="G161" s="9"/>
       <c r="H161" s="28"/>
     </row>
     <row r="162" ht="14.25" customHeight="1">
-      <c r="A162" s="1">
-        <v>46336.0</v>
-      </c>
-      <c r="B162" s="2" t="s">
-        <v>38</v>
+      <c r="A162" s="23">
+        <v>46335.0</v>
+      </c>
+      <c r="B162" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="C162" s="9">
-        <v>65.0</v>
+        <v>90.0</v>
       </c>
       <c r="G162" s="9"/>
       <c r="H162" s="28"/>
     </row>
     <row r="163" ht="14.25" customHeight="1">
-      <c r="A163" s="23">
-        <v>46337.0</v>
-      </c>
-      <c r="B163" s="8" t="s">
-        <v>43</v>
+      <c r="A163" s="1">
+        <v>46336.0</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C163" s="9">
-        <v>95.12</v>
+        <v>65.0</v>
       </c>
       <c r="G163" s="9"/>
       <c r="H163" s="28"/>
@@ -5429,23 +5429,23 @@
         <v>46337.0</v>
       </c>
       <c r="B164" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C164" s="9">
-        <v>50.0</v>
+        <v>95.12</v>
       </c>
       <c r="G164" s="9"/>
       <c r="H164" s="28"/>
     </row>
     <row r="165" ht="14.25" customHeight="1">
       <c r="A165" s="23">
-        <v>46338.0</v>
+        <v>46337.0</v>
       </c>
       <c r="B165" s="8" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="C165" s="9">
-        <v>981.95</v>
+        <v>50.0</v>
       </c>
       <c r="G165" s="9"/>
       <c r="H165" s="28"/>
@@ -5455,36 +5455,36 @@
         <v>46338.0</v>
       </c>
       <c r="B166" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C166" s="3">
-        <v>2831.4</v>
+        <v>25</v>
+      </c>
+      <c r="C166" s="9">
+        <v>981.95</v>
       </c>
       <c r="G166" s="9"/>
       <c r="H166" s="28"/>
     </row>
     <row r="167" ht="14.25" customHeight="1">
       <c r="A167" s="23">
-        <v>46342.0</v>
+        <v>46338.0</v>
       </c>
       <c r="B167" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C167" s="9">
-        <v>132.4</v>
+        <v>33</v>
+      </c>
+      <c r="C167" s="3">
+        <v>2831.4</v>
       </c>
       <c r="G167" s="9"/>
       <c r="H167" s="28"/>
     </row>
     <row r="168" ht="14.25" customHeight="1">
       <c r="A168" s="23">
-        <v>46346.0</v>
-      </c>
-      <c r="B168" s="2" t="s">
-        <v>23</v>
+        <v>46342.0</v>
+      </c>
+      <c r="B168" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="C168" s="9">
-        <v>5750.0</v>
+        <v>132.4</v>
       </c>
       <c r="G168" s="9"/>
       <c r="H168" s="28"/>
@@ -5493,115 +5493,115 @@
       <c r="A169" s="23">
         <v>46346.0</v>
       </c>
-      <c r="B169" s="8" t="s">
-        <v>40</v>
+      <c r="B169" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C169" s="9">
-        <v>113.31</v>
+        <v>5750.0</v>
       </c>
       <c r="G169" s="9"/>
       <c r="H169" s="28"/>
     </row>
     <row r="170" ht="14.25" customHeight="1">
-      <c r="A170" s="1">
-        <v>46358.0</v>
+      <c r="A170" s="23">
+        <v>46346.0</v>
       </c>
       <c r="B170" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C170" s="9">
-        <v>1880.0</v>
+        <v>113.31</v>
       </c>
       <c r="G170" s="9"/>
       <c r="H170" s="28"/>
     </row>
     <row r="171" ht="14.25" customHeight="1">
       <c r="A171" s="1">
-        <v>46360.0</v>
+        <v>46358.0</v>
       </c>
       <c r="B171" s="8" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="C171" s="9">
-        <v>950.0</v>
+        <v>1880.0</v>
       </c>
       <c r="G171" s="9"/>
       <c r="H171" s="28"/>
     </row>
     <row r="172" ht="14.25" customHeight="1">
-      <c r="A172" s="23">
-        <v>46363.0</v>
+      <c r="A172" s="1">
+        <v>46360.0</v>
       </c>
       <c r="B172" s="8" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C172" s="9">
-        <v>195.0</v>
+        <v>950.0</v>
       </c>
       <c r="G172" s="9"/>
       <c r="H172" s="28"/>
     </row>
     <row r="173" ht="14.25" customHeight="1">
-      <c r="A173" s="1">
-        <v>46364.0</v>
+      <c r="A173" s="23">
+        <v>46363.0</v>
       </c>
       <c r="B173" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C173" s="9">
-        <v>120.0</v>
+        <v>195.0</v>
       </c>
       <c r="G173" s="9"/>
       <c r="H173" s="28"/>
     </row>
     <row r="174" ht="14.25" customHeight="1">
-      <c r="A174" s="23">
-        <v>46365.0</v>
+      <c r="A174" s="1">
+        <v>46364.0</v>
       </c>
       <c r="B174" s="8" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="C174" s="9">
-        <v>50.0</v>
+        <v>120.0</v>
       </c>
       <c r="G174" s="9"/>
       <c r="H174" s="28"/>
     </row>
     <row r="175" ht="14.25" customHeight="1">
-      <c r="A175" s="1">
+      <c r="A175" s="23">
         <v>46365.0</v>
       </c>
       <c r="B175" s="8" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="C175" s="9">
-        <v>530.0</v>
+        <v>50.0</v>
       </c>
       <c r="G175" s="9"/>
       <c r="H175" s="28"/>
     </row>
     <row r="176" ht="14.25" customHeight="1">
       <c r="A176" s="1">
-        <v>46366.0</v>
-      </c>
-      <c r="B176" s="2" t="s">
-        <v>38</v>
+        <v>46365.0</v>
+      </c>
+      <c r="B176" s="8" t="s">
+        <v>62</v>
       </c>
       <c r="C176" s="9">
-        <v>65.0</v>
+        <v>530.0</v>
       </c>
       <c r="G176" s="9"/>
       <c r="H176" s="28"/>
     </row>
     <row r="177" ht="14.25" customHeight="1">
-      <c r="A177" s="23">
-        <v>46367.0</v>
-      </c>
-      <c r="B177" s="8" t="s">
-        <v>25</v>
+      <c r="A177" s="1">
+        <v>46366.0</v>
+      </c>
+      <c r="B177" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C177" s="9">
-        <v>981.95</v>
+        <v>65.0</v>
       </c>
       <c r="G177" s="9"/>
       <c r="H177" s="28"/>
@@ -5611,10 +5611,10 @@
         <v>46367.0</v>
       </c>
       <c r="B178" s="8" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="C178" s="9">
-        <v>95.12</v>
+        <v>981.95</v>
       </c>
       <c r="G178" s="9"/>
       <c r="H178" s="28"/>
@@ -5624,10 +5624,10 @@
         <v>46367.0</v>
       </c>
       <c r="B179" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C179" s="3">
-        <v>2831.4</v>
+        <v>43</v>
+      </c>
+      <c r="C179" s="9">
+        <v>95.12</v>
       </c>
       <c r="G179" s="9"/>
       <c r="H179" s="28"/>
@@ -5637,75 +5637,75 @@
         <v>46367.0</v>
       </c>
       <c r="B180" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C180" s="9">
-        <v>2900.0</v>
+        <v>33</v>
+      </c>
+      <c r="C180" s="3">
+        <v>2831.4</v>
       </c>
       <c r="G180" s="9"/>
       <c r="H180" s="28"/>
     </row>
     <row r="181" ht="14.25" customHeight="1">
       <c r="A181" s="23">
-        <v>46368.0</v>
+        <v>46367.0</v>
       </c>
       <c r="B181" s="8" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="C181" s="9">
-        <v>132.4</v>
+        <v>2900.0</v>
       </c>
       <c r="G181" s="9"/>
       <c r="H181" s="28"/>
     </row>
     <row r="182" ht="14.25" customHeight="1">
       <c r="A182" s="23">
-        <v>46376.0</v>
-      </c>
-      <c r="B182" s="2" t="s">
-        <v>23</v>
+        <v>46368.0</v>
+      </c>
+      <c r="B182" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="C182" s="9">
-        <v>6250.0</v>
+        <v>132.4</v>
       </c>
       <c r="G182" s="9"/>
       <c r="H182" s="28"/>
     </row>
     <row r="183" ht="14.25" customHeight="1">
       <c r="A183" s="23">
-        <v>46377.0</v>
-      </c>
-      <c r="B183" s="8" t="s">
-        <v>40</v>
+        <v>46376.0</v>
+      </c>
+      <c r="B183" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C183" s="9">
-        <v>113.31</v>
+        <v>6250.0</v>
       </c>
       <c r="G183" s="9"/>
       <c r="H183" s="28"/>
     </row>
     <row r="184" ht="14.25" customHeight="1">
       <c r="A184" s="23">
-        <v>46391.0</v>
+        <v>46377.0</v>
       </c>
       <c r="B184" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C184" s="9">
-        <v>2000.0</v>
+        <v>113.31</v>
       </c>
       <c r="G184" s="9"/>
       <c r="H184" s="28"/>
     </row>
     <row r="185" ht="14.25" customHeight="1">
       <c r="A185" s="23">
-        <v>46393.0</v>
+        <v>46391.0</v>
       </c>
       <c r="B185" s="8" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C185" s="9">
-        <v>281.1</v>
+        <v>2000.0</v>
       </c>
       <c r="G185" s="9"/>
       <c r="H185" s="28"/>
@@ -5715,101 +5715,101 @@
         <v>46393.0</v>
       </c>
       <c r="B186" s="8" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C186" s="9">
-        <v>950.0</v>
+        <v>281.1</v>
       </c>
       <c r="G186" s="9"/>
       <c r="H186" s="28"/>
     </row>
     <row r="187" ht="14.25" customHeight="1">
       <c r="A187" s="23">
-        <v>46395.0</v>
+        <v>46393.0</v>
       </c>
       <c r="B187" s="8" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C187" s="9">
-        <v>120.0</v>
+        <v>950.0</v>
       </c>
       <c r="G187" s="9"/>
       <c r="H187" s="28"/>
     </row>
     <row r="188" ht="14.25" customHeight="1">
-      <c r="A188" s="1">
-        <v>46397.0</v>
-      </c>
-      <c r="B188" s="2" t="s">
-        <v>38</v>
+      <c r="A188" s="23">
+        <v>46395.0</v>
+      </c>
+      <c r="B188" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="C188" s="9">
-        <v>65.0</v>
+        <v>120.0</v>
       </c>
       <c r="G188" s="9"/>
       <c r="H188" s="28"/>
     </row>
     <row r="189" ht="14.25" customHeight="1">
-      <c r="A189" s="23">
-        <v>46398.0</v>
-      </c>
-      <c r="B189" s="8" t="s">
-        <v>43</v>
+      <c r="A189" s="1">
+        <v>46397.0</v>
+      </c>
+      <c r="B189" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C189" s="9">
-        <v>105.37</v>
+        <v>65.0</v>
       </c>
       <c r="G189" s="9"/>
       <c r="H189" s="28"/>
     </row>
     <row r="190" ht="14.25" customHeight="1">
       <c r="A190" s="23">
-        <v>46399.0</v>
+        <v>46398.0</v>
       </c>
       <c r="B190" s="8" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="C190" s="9">
-        <v>983.13</v>
+        <v>105.37</v>
       </c>
       <c r="G190" s="9"/>
       <c r="H190" s="28"/>
     </row>
     <row r="191" ht="14.25" customHeight="1">
       <c r="A191" s="23">
-        <v>46400.0</v>
+        <v>46399.0</v>
       </c>
       <c r="B191" s="8" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="C191" s="9">
-        <v>50.0</v>
+        <v>983.13</v>
       </c>
       <c r="G191" s="9"/>
       <c r="H191" s="28"/>
     </row>
     <row r="192" ht="14.25" customHeight="1">
       <c r="A192" s="23">
-        <v>46403.0</v>
+        <v>46400.0</v>
       </c>
       <c r="B192" s="8" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="C192" s="9">
-        <v>135.89</v>
+        <v>50.0</v>
       </c>
       <c r="G192" s="9"/>
       <c r="H192" s="28"/>
     </row>
     <row r="193" ht="14.25" customHeight="1">
       <c r="A193" s="23">
-        <v>46407.0</v>
-      </c>
-      <c r="B193" s="2" t="s">
-        <v>23</v>
+        <v>46403.0</v>
+      </c>
+      <c r="B193" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="C193" s="9">
-        <v>7796.0</v>
+        <v>135.89</v>
       </c>
       <c r="G193" s="9"/>
       <c r="H193" s="28"/>
@@ -5818,37 +5818,37 @@
       <c r="A194" s="23">
         <v>46407.0</v>
       </c>
-      <c r="B194" s="8" t="s">
-        <v>40</v>
+      <c r="B194" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C194" s="9">
-        <v>102.36</v>
+        <v>7796.0</v>
       </c>
       <c r="G194" s="9"/>
       <c r="H194" s="28"/>
     </row>
     <row r="195" ht="14.25" customHeight="1">
       <c r="A195" s="23">
-        <v>46420.0</v>
+        <v>46407.0</v>
       </c>
       <c r="B195" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C195" s="9">
-        <v>1800.0</v>
+        <v>102.36</v>
       </c>
       <c r="G195" s="9"/>
       <c r="H195" s="28"/>
     </row>
     <row r="196" ht="14.25" customHeight="1">
       <c r="A196" s="23">
-        <v>46422.0</v>
+        <v>46420.0</v>
       </c>
       <c r="B196" s="8" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C196" s="9">
-        <v>195.05</v>
+        <v>1800.0</v>
       </c>
       <c r="G196" s="9"/>
       <c r="H196" s="28"/>
@@ -5858,51 +5858,50 @@
         <v>46422.0</v>
       </c>
       <c r="B197" s="8" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C197" s="9">
-        <v>950.0</v>
+        <v>195.05</v>
       </c>
       <c r="G197" s="9"/>
       <c r="H197" s="28"/>
     </row>
     <row r="198" ht="14.25" customHeight="1">
       <c r="A198" s="23">
-        <v>46426.0</v>
+        <v>46422.0</v>
       </c>
       <c r="B198" s="8" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C198" s="9">
-        <v>120.0</v>
+        <v>950.0</v>
       </c>
       <c r="G198" s="9"/>
       <c r="H198" s="28"/>
     </row>
     <row r="199" ht="14.25" customHeight="1">
-      <c r="A199" s="1">
-        <v>46428.0</v>
-      </c>
-      <c r="B199" s="2" t="s">
-        <v>38</v>
+      <c r="A199" s="23">
+        <v>46426.0</v>
+      </c>
+      <c r="B199" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="C199" s="9">
-        <v>65.0</v>
+        <v>120.0</v>
       </c>
       <c r="G199" s="9"/>
       <c r="H199" s="28"/>
     </row>
     <row r="200" ht="14.25" customHeight="1">
-      <c r="A200" s="23">
+      <c r="A200" s="1">
         <v>46428.0</v>
       </c>
-      <c r="B200" s="8" t="s">
-        <v>44</v>
+      <c r="B200" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C200" s="9">
-        <v>50.0</v>
-      </c>
-      <c r="E200" s="2"/>
+        <v>65.0</v>
+      </c>
       <c r="G200" s="9"/>
       <c r="H200" s="28"/>
     </row>
@@ -5911,36 +5910,37 @@
         <v>46428.0</v>
       </c>
       <c r="B201" s="8" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="C201" s="9">
-        <v>530.0</v>
-      </c>
+        <v>50.0</v>
+      </c>
+      <c r="E201" s="2"/>
       <c r="G201" s="9"/>
       <c r="H201" s="28"/>
     </row>
     <row r="202" ht="14.25" customHeight="1">
       <c r="A202" s="23">
-        <v>46429.0</v>
+        <v>46428.0</v>
       </c>
       <c r="B202" s="8" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="C202" s="9">
-        <v>95.12</v>
+        <v>530.0</v>
       </c>
       <c r="G202" s="9"/>
       <c r="H202" s="28"/>
     </row>
     <row r="203" ht="14.25" customHeight="1">
       <c r="A203" s="23">
-        <v>46430.0</v>
+        <v>46429.0</v>
       </c>
       <c r="B203" s="8" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="C203" s="9">
-        <v>981.95</v>
+        <v>95.12</v>
       </c>
       <c r="G203" s="9"/>
       <c r="H203" s="28"/>
@@ -5949,37 +5949,37 @@
       <c r="A204" s="23">
         <v>46430.0</v>
       </c>
-      <c r="B204" s="23" t="s">
-        <v>27</v>
+      <c r="B204" s="8" t="s">
+        <v>25</v>
       </c>
       <c r="C204" s="9">
-        <v>1407.65</v>
+        <v>981.95</v>
       </c>
       <c r="G204" s="9"/>
       <c r="H204" s="28"/>
     </row>
     <row r="205" ht="14.25" customHeight="1">
       <c r="A205" s="23">
-        <v>46433.0</v>
-      </c>
-      <c r="B205" s="8" t="s">
-        <v>29</v>
+        <v>46430.0</v>
+      </c>
+      <c r="B205" s="23" t="s">
+        <v>27</v>
       </c>
       <c r="C205" s="9">
-        <v>132.4</v>
+        <v>1407.65</v>
       </c>
       <c r="G205" s="9"/>
       <c r="H205" s="28"/>
     </row>
     <row r="206" ht="14.25" customHeight="1">
       <c r="A206" s="23">
-        <v>46437.0</v>
-      </c>
-      <c r="B206" s="2" t="s">
-        <v>23</v>
+        <v>46433.0</v>
+      </c>
+      <c r="B206" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="C206" s="9">
-        <v>6004.07</v>
+        <v>132.4</v>
       </c>
       <c r="G206" s="9"/>
       <c r="H206" s="28"/>
@@ -5988,11 +5988,11 @@
       <c r="A207" s="23">
         <v>46437.0</v>
       </c>
-      <c r="B207" s="8" t="s">
-        <v>40</v>
+      <c r="B207" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C207" s="9">
-        <v>113.31</v>
+        <v>6004.07</v>
       </c>
       <c r="G207" s="9"/>
       <c r="H207" s="28"/>
@@ -6002,10 +6002,10 @@
         <v>46437.0</v>
       </c>
       <c r="B208" s="8" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C208" s="9">
-        <v>2831.4</v>
+        <v>113.31</v>
       </c>
       <c r="G208" s="9"/>
       <c r="H208" s="28"/>
@@ -6015,36 +6015,36 @@
         <v>46437.0</v>
       </c>
       <c r="B209" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C209" s="9">
-        <v>460.0</v>
+        <v>2831.4</v>
       </c>
       <c r="G209" s="9"/>
       <c r="H209" s="28"/>
     </row>
     <row r="210" ht="14.25" customHeight="1">
-      <c r="A210" s="1">
-        <v>46448.0</v>
+      <c r="A210" s="23">
+        <v>46437.0</v>
       </c>
       <c r="B210" s="8" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="C210" s="9">
-        <v>1771.95</v>
+        <v>460.0</v>
       </c>
       <c r="G210" s="9"/>
       <c r="H210" s="28"/>
     </row>
     <row r="211" ht="14.25" customHeight="1">
       <c r="A211" s="1">
-        <v>46451.0</v>
+        <v>46448.0</v>
       </c>
       <c r="B211" s="8" t="s">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="C211" s="9">
-        <v>64.89</v>
+        <v>1771.95</v>
       </c>
       <c r="G211" s="9"/>
       <c r="H211" s="28"/>
@@ -6054,23 +6054,23 @@
         <v>46451.0</v>
       </c>
       <c r="B212" s="8" t="s">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="C212" s="9">
-        <v>141.8</v>
+        <v>64.89</v>
       </c>
       <c r="G212" s="9"/>
       <c r="H212" s="28"/>
     </row>
     <row r="213" ht="14.25" customHeight="1">
       <c r="A213" s="1">
-        <v>46452.0</v>
+        <v>46451.0</v>
       </c>
       <c r="B213" s="8" t="s">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="C213" s="9">
-        <v>136.15</v>
+        <v>141.8</v>
       </c>
       <c r="G213" s="9"/>
       <c r="H213" s="28"/>
@@ -6080,36 +6080,36 @@
         <v>46452.0</v>
       </c>
       <c r="B214" s="8" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C214" s="9">
-        <v>800.0</v>
+        <v>136.15</v>
       </c>
       <c r="G214" s="9"/>
       <c r="H214" s="28"/>
     </row>
     <row r="215" ht="14.25" customHeight="1">
       <c r="A215" s="1">
-        <v>46455.0</v>
+        <v>46452.0</v>
       </c>
       <c r="B215" s="8" t="s">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="C215" s="9">
-        <v>57.89</v>
+        <v>800.0</v>
       </c>
       <c r="G215" s="9"/>
       <c r="H215" s="28"/>
     </row>
     <row r="216" ht="14.25" customHeight="1">
       <c r="A216" s="1">
-        <v>46456.0</v>
-      </c>
-      <c r="B216" s="2" t="s">
-        <v>39</v>
+        <v>46455.0</v>
+      </c>
+      <c r="B216" s="8" t="s">
+        <v>42</v>
       </c>
       <c r="C216" s="9">
-        <v>1336.73</v>
+        <v>57.89</v>
       </c>
       <c r="G216" s="9"/>
       <c r="H216" s="28"/>
@@ -6119,23 +6119,23 @@
         <v>46456.0</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C217" s="9">
-        <v>65.0</v>
+        <v>1336.73</v>
       </c>
       <c r="G217" s="9"/>
       <c r="H217" s="28"/>
     </row>
     <row r="218" ht="14.25" customHeight="1">
       <c r="A218" s="1">
-        <v>46457.0</v>
-      </c>
-      <c r="B218" s="8" t="s">
-        <v>43</v>
+        <v>46456.0</v>
+      </c>
+      <c r="B218" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C218" s="9">
-        <v>86.15</v>
+        <v>65.0</v>
       </c>
       <c r="G218" s="9"/>
       <c r="H218" s="28"/>
@@ -6145,23 +6145,23 @@
         <v>46457.0</v>
       </c>
       <c r="B219" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C219" s="9">
-        <v>50.0</v>
+        <v>86.15</v>
       </c>
       <c r="G219" s="9"/>
       <c r="H219" s="28"/>
     </row>
     <row r="220" ht="14.25" customHeight="1">
-      <c r="A220" s="23">
-        <v>46458.0</v>
+      <c r="A220" s="1">
+        <v>46457.0</v>
       </c>
       <c r="B220" s="8" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="C220" s="9">
-        <v>981.22</v>
+        <v>50.0</v>
       </c>
       <c r="G220" s="9"/>
       <c r="H220" s="28"/>
@@ -6171,36 +6171,36 @@
         <v>46458.0</v>
       </c>
       <c r="B221" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C221" s="3">
-        <v>2831.4</v>
+        <v>25</v>
+      </c>
+      <c r="C221" s="9">
+        <v>981.22</v>
       </c>
       <c r="G221" s="9"/>
       <c r="H221" s="28"/>
     </row>
     <row r="222" ht="14.25" customHeight="1">
-      <c r="A222" s="1">
-        <v>46462.0</v>
+      <c r="A222" s="23">
+        <v>46458.0</v>
       </c>
       <c r="B222" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C222" s="9">
-        <v>132.4</v>
+        <v>33</v>
+      </c>
+      <c r="C222" s="3">
+        <v>2831.4</v>
       </c>
       <c r="G222" s="9"/>
       <c r="H222" s="28"/>
     </row>
     <row r="223" ht="14.25" customHeight="1">
       <c r="A223" s="1">
-        <v>46466.0</v>
-      </c>
-      <c r="B223" s="2" t="s">
-        <v>23</v>
+        <v>46462.0</v>
+      </c>
+      <c r="B223" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="C223" s="9">
-        <v>7494.55</v>
+        <v>132.4</v>
       </c>
       <c r="G223" s="9"/>
       <c r="H223" s="28"/>
@@ -6209,32 +6209,38 @@
       <c r="A224" s="1">
         <v>46466.0</v>
       </c>
-      <c r="B224" s="8" t="s">
-        <v>40</v>
+      <c r="B224" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C224" s="9">
-        <v>87.84</v>
+        <v>7494.55</v>
       </c>
       <c r="G224" s="9"/>
       <c r="H224" s="28"/>
     </row>
     <row r="225" ht="14.25" customHeight="1">
       <c r="A225" s="1">
-        <v>46477.0</v>
+        <v>46466.0</v>
       </c>
       <c r="B225" s="8" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C225" s="9">
-        <v>35.62</v>
+        <v>87.84</v>
       </c>
       <c r="G225" s="9"/>
       <c r="H225" s="28"/>
     </row>
     <row r="226" ht="14.25" customHeight="1">
-      <c r="A226" s="23"/>
-      <c r="B226" s="23"/>
-      <c r="C226" s="9"/>
+      <c r="A226" s="1">
+        <v>46477.0</v>
+      </c>
+      <c r="B226" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C226" s="9">
+        <v>35.62</v>
+      </c>
       <c r="G226" s="9"/>
       <c r="H226" s="28"/>
     </row>
@@ -6932,9 +6938,9 @@
       <c r="H325" s="28"/>
     </row>
     <row r="326" ht="14.25" customHeight="1">
-      <c r="A326" s="29"/>
-      <c r="B326" s="29"/>
-      <c r="C326" s="30"/>
+      <c r="A326" s="23"/>
+      <c r="B326" s="23"/>
+      <c r="C326" s="9"/>
       <c r="G326" s="9"/>
       <c r="H326" s="28"/>
     </row>
@@ -7464,7 +7470,11 @@
       <c r="H401" s="28"/>
     </row>
     <row r="402" ht="14.25" customHeight="1">
-      <c r="A402" s="23"/>
+      <c r="A402" s="29"/>
+      <c r="B402" s="29"/>
+      <c r="C402" s="30"/>
+      <c r="G402" s="9"/>
+      <c r="H402" s="28"/>
     </row>
     <row r="403" ht="14.25" customHeight="1">
       <c r="A403" s="23"/>
@@ -7535,7 +7545,9 @@
     <row r="425" ht="14.25" customHeight="1">
       <c r="A425" s="23"/>
     </row>
-    <row r="426" ht="15.75" customHeight="1"/>
+    <row r="426" ht="14.25" customHeight="1">
+      <c r="A426" s="23"/>
+    </row>
     <row r="427" ht="15.75" customHeight="1"/>
     <row r="428" ht="15.75" customHeight="1"/>
     <row r="429" ht="15.75" customHeight="1"/>
@@ -8124,14 +8136,15 @@
     <row r="1012" ht="15.75" customHeight="1"/>
     <row r="1013" ht="15.75" customHeight="1"/>
     <row r="1014" ht="15.75" customHeight="1"/>
+    <row r="1015" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$1:$E$225">
-    <sortState ref="A1:E225">
-      <sortCondition ref="E1:E225"/>
-      <sortCondition ref="A1:A225"/>
-      <sortCondition ref="B1:B225"/>
-      <sortCondition ref="C1:C225"/>
-      <sortCondition ref="D1:D225"/>
+  <autoFilter ref="$A$1:$E$226">
+    <sortState ref="A1:E226">
+      <sortCondition ref="E1:E226"/>
+      <sortCondition ref="A1:A226"/>
+      <sortCondition ref="B1:B226"/>
+      <sortCondition ref="C1:C226"/>
+      <sortCondition ref="D1:D226"/>
     </sortState>
   </autoFilter>
   <printOptions/>
@@ -11072,7 +11085,7 @@
       </c>
       <c r="K3" s="51">
         <f>SUM(B4:B123)</f>
-        <v>220901.1</v>
+        <v>221021.1</v>
       </c>
       <c r="M3" s="8" t="s">
         <v>126</v>
@@ -11151,7 +11164,7 @@
       </c>
       <c r="K5" s="51">
         <f>SUMIFS(D4:D123,A4:A123,"&lt;="&amp;EOMONTH(TODAY(),0)+1-1,A4:A123,"&lt;&gt;")</f>
-        <v>17116.42</v>
+        <v>16996.42</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="1">
@@ -11188,7 +11201,7 @@
       </c>
       <c r="K6" s="51">
         <f>G17</f>
-        <v>1168.97</v>
+        <v>1048.97</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="1">
@@ -11198,7 +11211,7 @@
       </c>
       <c r="B7" s="56">
         <f>IF($A7="","",SUMIFS('Todos os Gastos'!$C:$C,'Todos os Gastos'!$A:$A,"&gt;="&amp;$A7,'Todos os Gastos'!$A:$A,"&lt;"&amp;EDATE($A7,1)))</f>
-        <v>24317.36</v>
+        <v>24437.36</v>
       </c>
       <c r="C7" s="56">
         <f>IF($A7="","",SUMIFS('Inventário de Lotes'!$D:$D,'Inventário de Lotes'!$B:$B,"&gt;="&amp;$A7,'Inventário de Lotes'!$B:$B,"&lt;"&amp;EDATE($A7,1)))</f>
@@ -11206,11 +11219,11 @@
       </c>
       <c r="D7" s="56">
         <f t="shared" si="1"/>
-        <v>2233.3</v>
+        <v>2113.3</v>
       </c>
       <c r="E7" s="57">
         <f>IF($A7="","",COUNTIFS('Todos os Gastos'!$A:$A,"&gt;="&amp;$A7,'Todos os Gastos'!$A:$A,"&lt;"&amp;EDATE($A7,1)))</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F7" s="57">
         <f>IF($A7="","",COUNTIFS('Inventário de Lotes'!$B:$B,"&gt;="&amp;$A7,'Inventário de Lotes'!$B:$B,"&lt;"&amp;EDATE($A7,1)))</f>
@@ -11218,14 +11231,14 @@
       </c>
       <c r="G7" s="56">
         <f t="shared" si="2"/>
-        <v>17116.42</v>
+        <v>16996.42</v>
       </c>
       <c r="J7" s="50" t="s">
         <v>130</v>
       </c>
       <c r="K7" s="51">
         <f>SUMIFS(D4:D123,A4:A123,"&gt;="&amp;EOMONTH(TODAY(),-1)+1,A4:A123,"&lt;"&amp;EDATE(EOMONTH(TODAY(),-1)+1,1))</f>
-        <v>2233.3</v>
+        <v>2113.3</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
@@ -11255,14 +11268,14 @@
       </c>
       <c r="G8" s="53">
         <f t="shared" si="2"/>
-        <v>17752.24</v>
+        <v>17632.24</v>
       </c>
       <c r="J8" s="50" t="s">
         <v>131</v>
       </c>
       <c r="K8" s="51">
         <f>AVERAGEIF(D4:D123,"&lt;&gt;",D4:D123)</f>
-        <v>83.49785714</v>
+        <v>74.92642857</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="1">
@@ -11292,14 +11305,14 @@
       </c>
       <c r="G9" s="56">
         <f t="shared" si="2"/>
-        <v>17168.06</v>
+        <v>17048.06</v>
       </c>
       <c r="J9" s="50" t="s">
         <v>132</v>
       </c>
       <c r="K9" s="51">
         <f>MAX(B4:B123)</f>
-        <v>24317.36</v>
+        <v>24437.36</v>
       </c>
     </row>
     <row r="10" ht="15.0" customHeight="1">
@@ -11329,7 +11342,7 @@
       </c>
       <c r="G10" s="53">
         <f t="shared" si="2"/>
-        <v>16023.88</v>
+        <v>15903.88</v>
       </c>
       <c r="J10" s="50" t="s">
         <v>133</v>
@@ -11366,7 +11379,7 @@
       </c>
       <c r="G11" s="56">
         <f t="shared" si="2"/>
-        <v>14229.7</v>
+        <v>14109.7</v>
       </c>
       <c r="J11" s="50" t="s">
         <v>134</v>
@@ -11403,7 +11416,7 @@
       </c>
       <c r="G12" s="53">
         <f t="shared" si="2"/>
-        <v>12835.72</v>
+        <v>12715.72</v>
       </c>
       <c r="J12" s="50" t="s">
         <v>135</v>
@@ -11440,7 +11453,7 @@
       </c>
       <c r="G13" s="56">
         <f t="shared" si="2"/>
-        <v>11941.54</v>
+        <v>11821.54</v>
       </c>
     </row>
     <row r="14" ht="15.0" customHeight="1">
@@ -11470,7 +11483,7 @@
       </c>
       <c r="G14" s="53">
         <f t="shared" si="2"/>
-        <v>7527.36</v>
+        <v>7407.36</v>
       </c>
       <c r="J14" s="59"/>
     </row>
@@ -11501,7 +11514,7 @@
       </c>
       <c r="G15" s="56">
         <f t="shared" si="2"/>
-        <v>7618.51</v>
+        <v>7498.51</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1">
@@ -11531,7 +11544,7 @@
       </c>
       <c r="G16" s="53">
         <f t="shared" si="2"/>
-        <v>4562.56</v>
+        <v>4442.56</v>
       </c>
     </row>
     <row r="17" ht="15.0" customHeight="1">
@@ -11561,7 +11574,7 @@
       </c>
       <c r="G17" s="56">
         <f t="shared" si="2"/>
-        <v>1168.97</v>
+        <v>1048.97</v>
       </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">

</xml_diff>

<commit_message>
Atualiza dados financeiros e cache BCB para referencia 2026-05-13
</commit_message>
<xml_diff>
--- a/dados/dados_financeiros.xlsx
+++ b/dados/dados_financeiros.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2413" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2419" uniqueCount="427">
   <si>
     <t>Mês</t>
   </si>
@@ -1878,11 +1878,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="169851099"/>
-        <c:axId val="974873360"/>
+        <c:axId val="1589058995"/>
+        <c:axId val="1625498977"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="169851099"/>
+        <c:axId val="1589058995"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1934,10 +1934,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="974873360"/>
+        <c:crossAx val="1625498977"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="974873360"/>
+        <c:axId val="1625498977"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2001,7 +2001,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="169851099"/>
+        <c:crossAx val="1589058995"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2238,7 +2238,7 @@
         <n v="110.0"/>
         <n v="44.0"/>
         <n v="98.88"/>
-        <n v="980.86"/>
+        <n v="980.0"/>
         <n v="5372.0"/>
         <n v="113.31"/>
         <n v="580.0"/>
@@ -2263,6 +2263,7 @@
         <n v="7494.55"/>
         <n v="35.62"/>
         <n v="6350.0"/>
+        <n v="980.86"/>
         <m/>
       </sharedItems>
     </cacheField>
@@ -2409,6 +2410,7 @@
         <item x="108"/>
         <item x="109"/>
         <item x="110"/>
+        <item x="111"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -2756,7 +2758,7 @@
       </c>
       <c r="J3" s="8">
         <f>SUM(B:B)</f>
-        <v>258373.74</v>
+        <v>258372.88</v>
       </c>
       <c r="L3" s="9">
         <f>EOMONTH(MAX(MAX('Todos os Gastos'!$A:$A),MAX('Salários'!$B:$B)),-1)+1</f>
@@ -2837,7 +2839,7 @@
       </c>
       <c r="J5" s="8">
         <f>SUMIFS(D:D,A:A,"&lt;="&amp;EOMONTH(TODAY(),0)+1-1,A:A,"&lt;&gt;")</f>
-        <v>14031.01</v>
+        <v>14031.87</v>
       </c>
       <c r="L5" s="10">
         <v>46023.0</v>
@@ -2850,7 +2852,7 @@
       </c>
       <c r="B6" s="3">
         <f>IF($A6="","",SUMIFS('Todos os Gastos'!$C:$C,'Todos os Gastos'!$A:$A,"&gt;="&amp;$A6,'Todos os Gastos'!$A:$A,"&lt;"&amp;EDATE($A6,1)))</f>
-        <v>15447.25</v>
+        <v>15446.39</v>
       </c>
       <c r="C6" s="3">
         <f>IF($A6="","",SUMIFS('Salários'!$D:$D,'Salários'!$B:$B,"&gt;="&amp;$A6,'Salários'!$B:$B,"&lt;"&amp;EDATE($A6,1)))</f>
@@ -2858,7 +2860,7 @@
       </c>
       <c r="D6" s="3">
         <f t="shared" si="1"/>
-        <v>1769.47</v>
+        <v>1770.33</v>
       </c>
       <c r="E6" s="4">
         <f>IF($A6="","",COUNTIFS('Todos os Gastos'!$A:$A,"&gt;="&amp;$A6,'Todos os Gastos'!$A:$A,"&lt;"&amp;EDATE($A6,1)))</f>
@@ -2870,14 +2872,14 @@
       </c>
       <c r="G6" s="3">
         <f t="shared" si="2"/>
-        <v>14031.01</v>
+        <v>14031.87</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>13</v>
       </c>
       <c r="J6" s="8">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("INDEX(G:G, MAX(FILTER(ROW(G:G), G:G&lt;&gt;"""")))"),-2488.409999999987)</f>
-        <v>-2488.41</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("INDEX(G:G, MAX(FILTER(ROW(G:G), G:G&lt;&gt;"""")))"),-2487.5499999999865)</f>
+        <v>-2487.55</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="1">
@@ -2907,14 +2909,14 @@
       </c>
       <c r="G7" s="6">
         <f t="shared" si="2"/>
-        <v>14311.83</v>
+        <v>14312.69</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>14</v>
       </c>
       <c r="J7" s="8">
         <f>SUMIFS(D:D,A:A,"&gt;="&amp;EOMONTH(TODAY(),-1)+1,A:A,"&lt;"&amp;EDATE(EOMONTH(TODAY(),-1)+1,1))</f>
-        <v>1769.47</v>
+        <v>1770.33</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
@@ -2944,14 +2946,14 @@
       </c>
       <c r="G8" s="3">
         <f t="shared" si="2"/>
-        <v>13532.65</v>
+        <v>13533.51</v>
       </c>
       <c r="I8" s="7" t="s">
         <v>15</v>
       </c>
       <c r="J8" s="8">
         <f>AVERAGEIF(D:D,"&lt;&gt;",D:D)</f>
-        <v>-146.3770588</v>
+        <v>-146.3264706</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="1">
@@ -2981,7 +2983,7 @@
       </c>
       <c r="G9" s="6">
         <f t="shared" si="2"/>
-        <v>12111.67</v>
+        <v>12112.53</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>16</v>
@@ -3018,7 +3020,7 @@
       </c>
       <c r="G10" s="3">
         <f t="shared" si="2"/>
-        <v>10122.49</v>
+        <v>10123.35</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>17</v>
@@ -3055,7 +3057,7 @@
       </c>
       <c r="G11" s="6">
         <f t="shared" si="2"/>
-        <v>8533.51</v>
+        <v>8534.37</v>
       </c>
       <c r="I11" s="7" t="s">
         <v>18</v>
@@ -3092,7 +3094,7 @@
       </c>
       <c r="G12" s="3">
         <f t="shared" si="2"/>
-        <v>7444.33</v>
+        <v>7445.19</v>
       </c>
       <c r="I12" s="7" t="s">
         <v>19</v>
@@ -3129,7 +3131,7 @@
       </c>
       <c r="G13" s="6">
         <f t="shared" si="2"/>
-        <v>3235.15</v>
+        <v>3236.01</v>
       </c>
     </row>
     <row r="14" ht="15.0" customHeight="1">
@@ -3159,7 +3161,7 @@
       </c>
       <c r="G14" s="3">
         <f t="shared" si="2"/>
-        <v>6074.89</v>
+        <v>6075.75</v>
       </c>
     </row>
     <row r="15" ht="15.0" customHeight="1">
@@ -3189,7 +3191,7 @@
       </c>
       <c r="G15" s="6">
         <f t="shared" si="2"/>
-        <v>3003.99</v>
+        <v>3004.85</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1">
@@ -3219,7 +3221,7 @@
       </c>
       <c r="G16" s="3">
         <f t="shared" si="2"/>
-        <v>-177.13</v>
+        <v>-176.27</v>
       </c>
     </row>
     <row r="17" ht="15.0" customHeight="1">
@@ -3249,7 +3251,7 @@
       </c>
       <c r="G17" s="6">
         <f t="shared" si="2"/>
-        <v>-4530.18</v>
+        <v>-4529.32</v>
       </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">
@@ -3279,7 +3281,7 @@
       </c>
       <c r="G18" s="3">
         <f t="shared" si="2"/>
-        <v>-2488.41</v>
+        <v>-2487.55</v>
       </c>
     </row>
     <row r="19" ht="15.0" customHeight="1">
@@ -13995,23 +13997,27 @@
       <c r="H107" s="57"/>
     </row>
     <row r="108" ht="14.25" customHeight="1">
-      <c r="A108" s="34">
-        <v>46154.0</v>
+      <c r="A108" s="45">
+        <v>46155.0</v>
       </c>
       <c r="B108" s="43" t="s">
         <v>61</v>
       </c>
       <c r="C108" s="46">
-        <v>980.86</v>
-      </c>
-      <c r="D108" s="42"/>
-      <c r="E108" s="42"/>
+        <v>980.0</v>
+      </c>
+      <c r="D108" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="E108" s="58" t="s">
+        <v>53</v>
+      </c>
       <c r="G108" s="56"/>
       <c r="H108" s="57"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
-      <c r="A109" s="34">
-        <v>46154.0</v>
+      <c r="A109" s="45">
+        <v>46155.0</v>
       </c>
       <c r="B109" s="42" t="s">
         <v>67</v>
@@ -14019,14 +14025,18 @@
       <c r="C109" s="48">
         <v>2831.4</v>
       </c>
-      <c r="D109" s="42"/>
-      <c r="E109" s="42"/>
+      <c r="D109" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="E109" s="58" t="s">
+        <v>53</v>
+      </c>
       <c r="G109" s="56"/>
       <c r="H109" s="57"/>
     </row>
     <row r="110" ht="14.25" customHeight="1">
-      <c r="A110" s="34">
-        <v>46154.0</v>
+      <c r="A110" s="45">
+        <v>46155.0</v>
       </c>
       <c r="B110" s="43" t="s">
         <v>56</v>
@@ -14034,8 +14044,12 @@
       <c r="C110" s="48">
         <v>50.0</v>
       </c>
-      <c r="D110" s="42"/>
-      <c r="E110" s="42"/>
+      <c r="D110" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="E110" s="58" t="s">
+        <v>53</v>
+      </c>
       <c r="G110" s="56"/>
       <c r="H110" s="57"/>
     </row>

</xml_diff>

<commit_message>
Atualiza planilha de dados financeiros
</commit_message>
<xml_diff>
--- a/dados/dados_financeiros.xlsx
+++ b/dados/dados_financeiros.xlsx
@@ -1878,11 +1878,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1589058995"/>
-        <c:axId val="1625498977"/>
+        <c:axId val="2052730152"/>
+        <c:axId val="1414690732"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1589058995"/>
+        <c:axId val="2052730152"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1934,10 +1934,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1625498977"/>
+        <c:crossAx val="1414690732"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1625498977"/>
+        <c:axId val="1414690732"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2001,7 +2001,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1589058995"/>
+        <c:crossAx val="2052730152"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>

</xml_diff>

<commit_message>
dados: atualiza base financeira e cache BCB
</commit_message>
<xml_diff>
--- a/dados/dados_financeiros.xlsx
+++ b/dados/dados_financeiros.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2427" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2429" uniqueCount="427">
   <si>
     <t>Mês</t>
   </si>
@@ -1881,11 +1881,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1812406660"/>
-        <c:axId val="130072092"/>
+        <c:axId val="884757071"/>
+        <c:axId val="1327428171"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1812406660"/>
+        <c:axId val="884757071"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1937,10 +1937,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="130072092"/>
+        <c:crossAx val="1327428171"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="130072092"/>
+        <c:axId val="1327428171"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2004,7 +2004,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1812406660"/>
+        <c:crossAx val="884757071"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -14110,8 +14110,12 @@
       <c r="C113" s="49">
         <v>132.4</v>
       </c>
-      <c r="D113" s="42"/>
-      <c r="E113" s="42"/>
+      <c r="D113" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="E113" s="59" t="s">
+        <v>45</v>
+      </c>
       <c r="G113" s="57"/>
       <c r="H113" s="58"/>
     </row>

</xml_diff>

<commit_message>
ME-PRE-ETAPA5-01: atualiza contrato e dados operacionais
</commit_message>
<xml_diff>
--- a/dados/dados_financeiros.xlsx
+++ b/dados/dados_financeiros.xlsx
@@ -1881,11 +1881,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="427096795"/>
-        <c:axId val="1732889436"/>
+        <c:axId val="1048450435"/>
+        <c:axId val="1683088026"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="427096795"/>
+        <c:axId val="1048450435"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1937,10 +1937,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1732889436"/>
+        <c:crossAx val="1683088026"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1732889436"/>
+        <c:axId val="1683088026"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2004,7 +2004,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="427096795"/>
+        <c:crossAx val="1048450435"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2250,6 +2250,8 @@
         <n v="73.19"/>
         <n v="19.02"/>
         <n v="580.0"/>
+        <n v="101.47"/>
+        <n v="983.8"/>
         <n v="7200.0"/>
         <n v="113.31"/>
         <n v="930.0"/>
@@ -2431,6 +2433,8 @@
         <item x="116"/>
         <item x="117"/>
         <item x="118"/>
+        <item x="119"/>
+        <item x="120"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -2781,7 +2785,7 @@
       </c>
       <c r="J3" s="8">
         <f>SUM(B:B)</f>
-        <v>258704.46</v>
+        <v>258712.66</v>
       </c>
       <c r="L3" s="9">
         <f>EOMONTH(MAX(MAX('Todos os Gastos'!$A:$A),MAX('Salários'!$B:$B)),-1)+1</f>
@@ -2822,7 +2826,7 @@
       </c>
       <c r="J4" s="8">
         <f>SUM(C:C)</f>
-        <v>255885.33</v>
+        <v>258648.33</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>11</v>
@@ -2901,8 +2905,8 @@
         <v>13</v>
       </c>
       <c r="J6" s="8">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("INDEX(G:G, MAX(FILTER(ROW(G:G), G:G&lt;&gt;"""")))"),-2819.1299999999883)</f>
-        <v>-2819.13</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("INDEX(G:G, MAX(FILTER(ROW(G:G), G:G&lt;&gt;"""")))"),-64.3299999999872)</f>
+        <v>-64.33</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="1">
@@ -2912,15 +2916,15 @@
       </c>
       <c r="B7" s="6">
         <f>IF($A7="","",SUMIFS('Todos os Gastos'!$C:$C,'Todos os Gastos'!$A:$A,"&gt;="&amp;$A7,'Todos os Gastos'!$A:$A,"&lt;"&amp;EDATE($A7,1)))</f>
-        <v>14599.18</v>
+        <v>14607.38</v>
       </c>
       <c r="C7" s="6">
         <f>IF($A7="","",SUMIFS('Salários'!$D:$D,'Salários'!$B:$B,"&gt;="&amp;$A7,'Salários'!$B:$B,"&lt;"&amp;EDATE($A7,1)))</f>
-        <v>14480</v>
+        <v>17243</v>
       </c>
       <c r="D7" s="6">
         <f t="shared" si="1"/>
-        <v>-119.18</v>
+        <v>2635.62</v>
       </c>
       <c r="E7" s="4">
         <f>IF($A7="","",COUNTIFS('Todos os Gastos'!$A:$A,"&gt;="&amp;$A7,'Todos os Gastos'!$A:$A,"&lt;"&amp;EDATE($A7,1)))</f>
@@ -2932,7 +2936,7 @@
       </c>
       <c r="G7" s="6">
         <f t="shared" si="2"/>
-        <v>13981.11</v>
+        <v>16735.91</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>14</v>
@@ -2969,14 +2973,14 @@
       </c>
       <c r="G8" s="3">
         <f t="shared" si="2"/>
-        <v>13201.93</v>
+        <v>15956.73</v>
       </c>
       <c r="I8" s="7" t="s">
         <v>15</v>
       </c>
       <c r="J8" s="8">
         <f>AVERAGEIF(D:D,"&lt;&gt;",D:D)</f>
-        <v>-165.8311765</v>
+        <v>-3.784117647</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="1">
@@ -3006,7 +3010,7 @@
       </c>
       <c r="G9" s="6">
         <f t="shared" si="2"/>
-        <v>11780.95</v>
+        <v>14535.75</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>16</v>
@@ -3043,7 +3047,7 @@
       </c>
       <c r="G10" s="3">
         <f t="shared" si="2"/>
-        <v>9791.77</v>
+        <v>12546.57</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>17</v>
@@ -3080,7 +3084,7 @@
       </c>
       <c r="G11" s="6">
         <f t="shared" si="2"/>
-        <v>8202.79</v>
+        <v>10957.59</v>
       </c>
       <c r="I11" s="7" t="s">
         <v>18</v>
@@ -3117,7 +3121,7 @@
       </c>
       <c r="G12" s="3">
         <f t="shared" si="2"/>
-        <v>7113.61</v>
+        <v>9868.41</v>
       </c>
       <c r="I12" s="7" t="s">
         <v>19</v>
@@ -3154,7 +3158,7 @@
       </c>
       <c r="G13" s="6">
         <f t="shared" si="2"/>
-        <v>2904.43</v>
+        <v>5659.23</v>
       </c>
     </row>
     <row r="14" ht="15.0" customHeight="1">
@@ -3184,7 +3188,7 @@
       </c>
       <c r="G14" s="3">
         <f t="shared" si="2"/>
-        <v>5744.17</v>
+        <v>8498.97</v>
       </c>
     </row>
     <row r="15" ht="15.0" customHeight="1">
@@ -3214,7 +3218,7 @@
       </c>
       <c r="G15" s="6">
         <f t="shared" si="2"/>
-        <v>2673.27</v>
+        <v>5428.07</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1">
@@ -3244,7 +3248,7 @@
       </c>
       <c r="G16" s="3">
         <f t="shared" si="2"/>
-        <v>-507.85</v>
+        <v>2246.95</v>
       </c>
     </row>
     <row r="17" ht="15.0" customHeight="1">
@@ -3274,7 +3278,7 @@
       </c>
       <c r="G17" s="6">
         <f t="shared" si="2"/>
-        <v>-4860.9</v>
+        <v>-2106.1</v>
       </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">
@@ -3304,7 +3308,7 @@
       </c>
       <c r="G18" s="3">
         <f t="shared" si="2"/>
-        <v>-2819.13</v>
+        <v>-64.33</v>
       </c>
     </row>
     <row r="19" ht="15.0" customHeight="1">
@@ -7556,8 +7560,8 @@
       <c r="C19" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="28">
-        <v>7000.0</v>
+      <c r="D19" s="26">
+        <v>7663.0</v>
       </c>
     </row>
     <row r="20">
@@ -7571,7 +7575,7 @@
         <v>26</v>
       </c>
       <c r="D20" s="26">
-        <v>1800.0</v>
+        <v>3900.0</v>
       </c>
     </row>
     <row r="21">
@@ -14315,8 +14319,8 @@
       <c r="B125" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="C125" s="49">
-        <v>95.12</v>
+      <c r="C125" s="47">
+        <v>101.47</v>
       </c>
       <c r="D125" s="42"/>
       <c r="E125" s="42"/>
@@ -14330,8 +14334,8 @@
       <c r="B126" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="C126" s="49">
-        <v>981.95</v>
+      <c r="C126" s="47">
+        <v>983.8</v>
       </c>
       <c r="D126" s="42"/>
       <c r="E126" s="42"/>

</xml_diff>

<commit_message>
Atualiza dados financeiros operacionais
</commit_message>
<xml_diff>
--- a/dados/dados_financeiros.xlsx
+++ b/dados/dados_financeiros.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2447" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2451" uniqueCount="430">
   <si>
     <t>Mês</t>
   </si>
@@ -324,6 +324,9 @@
     <t>Futebol</t>
   </si>
   <si>
+    <t>Lote 7600 jun.</t>
+  </si>
+  <si>
     <t>Mari</t>
   </si>
   <si>
@@ -394,9 +397,6 @@
   </si>
   <si>
     <t>Lote 3400 mai.</t>
-  </si>
-  <si>
-    <t>Lote 7600 jun.</t>
   </si>
   <si>
     <t>Taxa_Base_CDI</t>
@@ -1890,11 +1890,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1221299180"/>
-        <c:axId val="50444089"/>
+        <c:axId val="1505083291"/>
+        <c:axId val="2090637336"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1221299180"/>
+        <c:axId val="1505083291"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1946,10 +1946,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50444089"/>
+        <c:crossAx val="2090637336"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50444089"/>
+        <c:axId val="2090637336"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2013,7 +2013,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1221299180"/>
+        <c:crossAx val="1505083291"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2311,6 +2311,7 @@
         <s v="Lote 190 mai"/>
         <s v="Lote 3120 mai"/>
         <s v="Lote 2800 mai."/>
+        <s v="Lote 7600 jun."/>
         <m/>
       </sharedItems>
     </cacheField>
@@ -2458,7 +2459,7 @@
     </pivotField>
     <pivotField name="Lote usado" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
       <items>
-        <item h="1" x="14"/>
+        <item h="1" x="15"/>
         <item x="1"/>
         <item x="11"/>
         <item x="2"/>
@@ -2471,6 +2472,7 @@
         <item x="7"/>
         <item x="6"/>
         <item x="9"/>
+        <item h="1" x="14"/>
         <item x="8"/>
         <item x="0"/>
         <item t="default"/>
@@ -14247,8 +14249,12 @@
       <c r="C119" s="47">
         <v>5301.28</v>
       </c>
-      <c r="D119" s="42"/>
-      <c r="E119" s="42"/>
+      <c r="D119" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="E119" s="59" t="s">
+        <v>97</v>
+      </c>
       <c r="G119" s="57"/>
       <c r="H119" s="58"/>
     </row>
@@ -14262,8 +14268,12 @@
       <c r="C120" s="47">
         <v>400.0</v>
       </c>
-      <c r="D120" s="35"/>
-      <c r="E120" s="35"/>
+      <c r="D120" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="E120" s="59" t="s">
+        <v>97</v>
+      </c>
       <c r="G120" s="57"/>
       <c r="H120" s="58"/>
     </row>
@@ -14332,7 +14342,7 @@
         <v>46183.0</v>
       </c>
       <c r="B125" s="43" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C125" s="47">
         <v>50.0</v>
@@ -14452,7 +14462,7 @@
         <v>46192.0</v>
       </c>
       <c r="B133" s="37" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C133" s="47">
         <v>40.0</v>
@@ -14968,7 +14978,7 @@
         <v>46273.0</v>
       </c>
       <c r="B167" s="42" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C167" s="49">
         <v>90.0</v>
@@ -15178,7 +15188,7 @@
         <v>46303.0</v>
       </c>
       <c r="B181" s="42" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C181" s="49">
         <v>90.0</v>
@@ -15193,7 +15203,7 @@
         <v>46303.0</v>
       </c>
       <c r="B182" s="42" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C182" s="49">
         <v>119.8</v>
@@ -15388,7 +15398,7 @@
         <v>46335.0</v>
       </c>
       <c r="B195" s="42" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C195" s="49">
         <v>90.0</v>
@@ -15628,7 +15638,7 @@
         <v>46367.0</v>
       </c>
       <c r="B211" s="42" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C211" s="49">
         <v>2900.0</v>
@@ -20014,27 +20024,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="21" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C1" s="21" t="s">
         <v>21</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="66" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B2" s="59" t="s">
         <v>46</v>
@@ -20049,15 +20059,15 @@
         <v>3122.53</v>
       </c>
       <c r="F2" s="67" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="66" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B3" s="59" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C3" s="27">
         <v>46146.0</v>
@@ -20069,7 +20079,7 @@
         <v>3119.0</v>
       </c>
       <c r="F3" s="67" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
@@ -20077,7 +20087,7 @@
         <v>61</v>
       </c>
       <c r="B4" s="59" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C4" s="27">
         <v>46148.0</v>
@@ -20089,7 +20099,7 @@
         <v>3000.0</v>
       </c>
       <c r="F4" s="67" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -20109,7 +20119,7 @@
         <v>192.41</v>
       </c>
       <c r="F5" s="67" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6">
@@ -24115,19 +24125,19 @@
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B1" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
@@ -24144,7 +24154,7 @@
         <v>4000.0</v>
       </c>
       <c r="E2" s="70" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
@@ -24161,7 +24171,7 @@
         <v>6630.64</v>
       </c>
       <c r="E3" s="70" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
@@ -24178,7 +24188,7 @@
         <v>10342.0</v>
       </c>
       <c r="E4" s="70" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -24195,7 +24205,7 @@
         <v>4124.75</v>
       </c>
       <c r="E5" s="70" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
@@ -24212,7 +24222,7 @@
         <v>5400.0</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
@@ -24229,12 +24239,12 @@
         <v>2063.11</v>
       </c>
       <c r="E7" s="70" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="66" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B8" s="71">
         <v>46084.0</v>
@@ -24246,12 +24256,12 @@
         <v>3000.0</v>
       </c>
       <c r="E8" s="73" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="66" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B9" s="71">
         <v>46085.0</v>
@@ -24263,7 +24273,7 @@
         <v>3000.0</v>
       </c>
       <c r="E9" s="73" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1">
@@ -24280,7 +24290,7 @@
         <v>8587.0</v>
       </c>
       <c r="E10" s="74" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -24297,7 +24307,7 @@
         <v>5680.0</v>
       </c>
       <c r="E11" s="67" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -24314,7 +24324,7 @@
         <v>7536.72</v>
       </c>
       <c r="E12" s="67" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1">
@@ -24331,12 +24341,12 @@
         <v>2800.0</v>
       </c>
       <c r="E13" s="67" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="59" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B14" s="27">
         <v>46150.0</v>
@@ -24348,12 +24358,12 @@
         <v>3000.0</v>
       </c>
       <c r="E14" s="67" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="59" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B15" s="27">
         <v>46150.0</v>
@@ -24365,12 +24375,12 @@
         <v>3429.0</v>
       </c>
       <c r="E15" s="67" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="59" t="s">
-        <v>121</v>
+        <v>97</v>
       </c>
       <c r="B16" s="27">
         <v>46174.0</v>
@@ -24382,7 +24392,7 @@
         <v>7561.0</v>
       </c>
       <c r="E16" s="67" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -31275,7 +31285,7 @@
     </row>
     <row r="18">
       <c r="A18" s="82" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B18" s="83">
         <v>120.0</v>
@@ -35626,7 +35636,7 @@
     </row>
     <row r="49">
       <c r="A49" s="82" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B49" s="83">
         <v>150.0</v>
@@ -36873,7 +36883,7 @@
     </row>
     <row r="58">
       <c r="A58" s="82" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B58" s="83">
         <v>105.0</v>
@@ -37014,7 +37024,7 @@
     </row>
     <row r="59">
       <c r="A59" s="82" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B59" s="83">
         <v>103.0</v>
@@ -37282,7 +37292,7 @@
     </row>
     <row r="61">
       <c r="A61" s="82" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B61" s="83">
         <v>230.0</v>
@@ -40815,7 +40825,7 @@
     </row>
     <row r="86">
       <c r="A86" s="82" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B86" s="83">
         <v>220.0</v>

</xml_diff>

<commit_message>
Atualiza dados financeiros e cache da execução
</commit_message>
<xml_diff>
--- a/dados/dados_financeiros.xlsx
+++ b/dados/dados_financeiros.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2453" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2457" uniqueCount="431">
   <si>
     <t>Mês</t>
   </si>
@@ -111,9 +111,6 @@
     <t>Salário UFV</t>
   </si>
   <si>
-    <t>Salário UEMG</t>
-  </si>
-  <si>
     <t>Velt</t>
   </si>
   <si>
@@ -121,6 +118,9 @@
   </si>
   <si>
     <t>Bolsa Doutorado</t>
+  </si>
+  <si>
+    <t>Salário UEMG</t>
   </si>
   <si>
     <t/>
@@ -1899,11 +1899,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="796605436"/>
-        <c:axId val="1688745908"/>
+        <c:axId val="1997471734"/>
+        <c:axId val="1112197495"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="796605436"/>
+        <c:axId val="1997471734"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1955,10 +1955,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1688745908"/>
+        <c:crossAx val="1112197495"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1688745908"/>
+        <c:axId val="1112197495"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2022,7 +2022,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="796605436"/>
+        <c:crossAx val="1997471734"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -7350,21 +7350,21 @@
     </row>
     <row r="3">
       <c r="A3" s="22" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B3" s="23">
         <v>46027.0</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D3" s="24">
-        <v>3634.7</v>
+        <v>5680.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4" s="23">
         <v>46027.0</v>
@@ -7373,12 +7373,12 @@
         <v>28</v>
       </c>
       <c r="D4" s="24">
-        <v>5680.0</v>
+        <v>4500.0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="22" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B5" s="23">
         <v>46027.0</v>
@@ -7387,7 +7387,7 @@
         <v>29</v>
       </c>
       <c r="D5" s="24">
-        <v>4500.0</v>
+        <v>3634.7</v>
       </c>
     </row>
     <row r="6">
@@ -7406,21 +7406,21 @@
     </row>
     <row r="7">
       <c r="A7" s="22" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B7" s="25">
         <v>46058.0</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" s="24">
-        <v>2063.11</v>
+        <v>11360.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B8" s="25">
         <v>46058.0</v>
@@ -7429,12 +7429,12 @@
         <v>28</v>
       </c>
       <c r="D8" s="24">
-        <v>11360.0</v>
+        <v>4500.0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="22" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B9" s="25">
         <v>46058.0</v>
@@ -7443,7 +7443,7 @@
         <v>29</v>
       </c>
       <c r="D9" s="24">
-        <v>4500.0</v>
+        <v>2063.11</v>
       </c>
     </row>
     <row r="10">
@@ -7462,30 +7462,30 @@
     </row>
     <row r="11">
       <c r="A11" s="22" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B11" s="25">
         <v>46087.0</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D11" s="24">
-        <v>3523.0</v>
+        <v>5680.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="22" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B12" s="25">
         <v>46087.0</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D12" s="24">
-        <v>5680.0</v>
+        <v>3523.0</v>
       </c>
     </row>
     <row r="13">
@@ -7504,30 +7504,30 @@
     </row>
     <row r="14">
       <c r="A14" s="22" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B14" s="25">
         <v>46120.0</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D14" s="24">
-        <v>3696.0</v>
+        <v>5680.0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="22" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B15" s="25">
         <v>46120.0</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D15" s="24">
-        <v>5680.0</v>
+        <v>3696.0</v>
       </c>
     </row>
     <row r="16">
@@ -7546,30 +7546,30 @@
     </row>
     <row r="17">
       <c r="A17" s="22" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B17" s="25">
         <v>46150.0</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D17" s="24">
-        <v>3900.0</v>
+        <v>5680.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="22" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B18" s="25">
         <v>46150.0</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D18" s="24">
-        <v>5680.0</v>
+        <v>3900.0</v>
       </c>
     </row>
     <row r="19">
@@ -7588,30 +7588,30 @@
     </row>
     <row r="20">
       <c r="A20" s="22" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B20" s="28">
         <v>46178.0</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="D20" s="26">
-        <v>3900.0</v>
+        <v>27</v>
+      </c>
+      <c r="D20" s="29">
+        <v>5680.0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="28">
-        <v>46178.0</v>
+        <v>24</v>
+      </c>
+      <c r="B21" s="27">
+        <v>46181.0</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="29">
-        <v>5680.0</v>
+        <v>29</v>
+      </c>
+      <c r="D21" s="26">
+        <v>3900.0</v>
       </c>
     </row>
     <row r="22">
@@ -7630,13 +7630,13 @@
     </row>
     <row r="23">
       <c r="A23" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B23" s="28">
         <v>46208.0</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D23" s="29">
         <v>5680.0</v>
@@ -7661,13 +7661,13 @@
     </row>
     <row r="25">
       <c r="A25" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B25" s="28">
         <v>46238.0</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D25" s="29">
         <v>5680.0</v>
@@ -7689,13 +7689,13 @@
     </row>
     <row r="27">
       <c r="A27" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27" s="28">
         <v>46269.0</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D27" s="29">
         <v>5680.0</v>
@@ -7717,13 +7717,13 @@
     </row>
     <row r="29">
       <c r="A29" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B29" s="28">
         <v>46300.0</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D29" s="29">
         <v>5680.0</v>
@@ -7745,13 +7745,13 @@
     </row>
     <row r="31">
       <c r="A31" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B31" s="28">
         <v>46331.0</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D31" s="29">
         <v>5680.0</v>
@@ -7773,13 +7773,13 @@
     </row>
     <row r="33">
       <c r="A33" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B33" s="28">
         <v>46362.0</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D33" s="29">
         <v>5680.0</v>
@@ -7801,13 +7801,13 @@
     </row>
     <row r="35">
       <c r="A35" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B35" s="23">
         <v>46392.0</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D35" s="24">
         <v>5680.0</v>
@@ -7829,13 +7829,13 @@
     </row>
     <row r="37">
       <c r="A37" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B37" s="28">
         <v>46424.0</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D37" s="29">
         <v>5680.0</v>
@@ -7857,13 +7857,13 @@
     </row>
     <row r="39">
       <c r="A39" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B39" s="28">
         <v>46452.0</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D39" s="29">
         <v>5680.0</v>
@@ -7885,13 +7885,13 @@
     </row>
     <row r="41">
       <c r="A41" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B41" s="27">
         <v>46483.0</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D41" s="29">
         <v>5680.0</v>
@@ -7913,13 +7913,13 @@
     </row>
     <row r="43">
       <c r="A43" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B43" s="27">
         <v>46513.0</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D43" s="29">
         <v>5680.0</v>
@@ -11773,6 +11773,7 @@
   <autoFilter ref="$A$1:$D$43">
     <sortState ref="A1:D43">
       <sortCondition ref="B1:B43"/>
+      <sortCondition ref="C1:C43"/>
       <sortCondition ref="A1:A43"/>
     </sortState>
   </autoFilter>
@@ -13194,7 +13195,7 @@
         <v>46101.0</v>
       </c>
       <c r="B65" s="42" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C65" s="49">
         <v>75.0</v>
@@ -13645,7 +13646,7 @@
         <v>46126.0</v>
       </c>
       <c r="B87" s="42" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C87" s="47">
         <v>18.75</v>
@@ -14296,8 +14297,12 @@
       <c r="C121" s="49">
         <v>950.0</v>
       </c>
-      <c r="D121" s="42"/>
-      <c r="E121" s="42"/>
+      <c r="D121" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="E121" s="59" t="s">
+        <v>97</v>
+      </c>
       <c r="G121" s="57"/>
       <c r="H121" s="58"/>
     </row>
@@ -14311,8 +14316,12 @@
       <c r="C122" s="47">
         <v>110.0</v>
       </c>
-      <c r="D122" s="42"/>
-      <c r="E122" s="42"/>
+      <c r="D122" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="E122" s="59" t="s">
+        <v>97</v>
+      </c>
       <c r="G122" s="57"/>
       <c r="H122" s="58"/>
     </row>

</xml_diff>

<commit_message>
Atualiza dados financeiros e cache BCB após ME-526
</commit_message>
<xml_diff>
--- a/dados/dados_financeiros.xlsx
+++ b/dados/dados_financeiros.xlsx
@@ -1917,11 +1917,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1066563110"/>
-        <c:axId val="600694185"/>
+        <c:axId val="1465629420"/>
+        <c:axId val="1652203528"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1066563110"/>
+        <c:axId val="1465629420"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1973,10 +1973,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="600694185"/>
+        <c:crossAx val="1652203528"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="600694185"/>
+        <c:axId val="1652203528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2040,7 +2040,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1066563110"/>
+        <c:crossAx val="1465629420"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="J5" s="8">
         <f>SUMIFS(D:D,A:A,"&lt;="&amp;EOMONTH(TODAY(),0)+1-1,A:A,"&lt;&gt;")</f>
-        <v>13415.75</v>
+        <v>13945.75</v>
       </c>
       <c r="L5" s="10">
         <v>46023.0</v>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="B7" s="6">
         <f>IF($A7="","",SUMIFS('Todos os Gastos'!$C:$C,'Todos os Gastos'!$A:$A,"&gt;="&amp;$A7,'Todos os Gastos'!$A:$A,"&lt;"&amp;EDATE($A7,1)))</f>
-        <v>17822.54</v>
+        <v>17292.54</v>
       </c>
       <c r="C7" s="6">
         <f>IF($A7="","",SUMIFS('Salários'!$D:$D,'Salários'!$B:$B,"&gt;="&amp;$A7,'Salários'!$B:$B,"&lt;"&amp;EDATE($A7,1)))</f>
@@ -2984,11 +2984,11 @@
       </c>
       <c r="D7" s="6">
         <f t="shared" si="1"/>
-        <v>-679.54</v>
+        <v>-149.54</v>
       </c>
       <c r="E7" s="4">
         <f>IF($A7="","",COUNTIFS('Todos os Gastos'!$A:$A,"&gt;="&amp;$A7,'Todos os Gastos'!$A:$A,"&lt;"&amp;EDATE($A7,1)))</f>
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F7" s="4">
         <f>IF($A7="","",COUNTIFS('Salários'!$B:$B,"&gt;="&amp;$A7,'Salários'!$B:$B,"&lt;"&amp;EDATE($A7,1)))</f>
@@ -2996,14 +2996,14 @@
       </c>
       <c r="G7" s="6">
         <f t="shared" si="2"/>
-        <v>13415.75</v>
+        <v>13945.75</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>14</v>
       </c>
       <c r="J7" s="8">
         <f>SUMIFS(D:D,A:A,"&gt;="&amp;EOMONTH(TODAY(),-1)+1,A:A,"&lt;"&amp;EDATE(EOMONTH(TODAY(),-1)+1,1))</f>
-        <v>-679.54</v>
+        <v>-149.54</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="B8" s="3">
         <f>IF($A8="","",SUMIFS('Todos os Gastos'!$C:$C,'Todos os Gastos'!$A:$A,"&gt;="&amp;$A8,'Todos os Gastos'!$A:$A,"&lt;"&amp;EDATE($A8,1)))</f>
-        <v>13969.11</v>
+        <v>14499.11</v>
       </c>
       <c r="C8" s="3">
         <f>IF($A8="","",SUMIFS('Salários'!$D:$D,'Salários'!$B:$B,"&gt;="&amp;$A8,'Salários'!$B:$B,"&lt;"&amp;EDATE($A8,1)))</f>
@@ -3021,11 +3021,11 @@
       </c>
       <c r="D8" s="3">
         <f t="shared" si="1"/>
-        <v>-1289.11</v>
+        <v>-1819.11</v>
       </c>
       <c r="E8" s="4">
         <f>IF($A8="","",COUNTIFS('Todos os Gastos'!$A:$A,"&gt;="&amp;$A8,'Todos os Gastos'!$A:$A,"&lt;"&amp;EDATE($A8,1)))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F8" s="4">
         <f>IF($A8="","",COUNTIFS('Salários'!$B:$B,"&gt;="&amp;$A8,'Salários'!$B:$B,"&lt;"&amp;EDATE($A8,1)))</f>
@@ -14637,14 +14637,14 @@
       <c r="H137" s="58"/>
     </row>
     <row r="138" ht="14.25" customHeight="1">
-      <c r="A138" s="46">
-        <v>46192.0</v>
-      </c>
-      <c r="B138" s="42" t="s">
-        <v>66</v>
-      </c>
-      <c r="C138" s="49">
-        <v>530.0</v>
+      <c r="A138" s="34">
+        <v>46193.0</v>
+      </c>
+      <c r="B138" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="C138" s="47">
+        <v>5931.43</v>
       </c>
       <c r="D138" s="42"/>
       <c r="E138" s="42"/>
@@ -14652,14 +14652,14 @@
       <c r="H138" s="58"/>
     </row>
     <row r="139" ht="14.25" customHeight="1">
-      <c r="A139" s="34">
+      <c r="A139" s="46">
         <v>46193.0</v>
       </c>
-      <c r="B139" s="35" t="s">
-        <v>36</v>
-      </c>
-      <c r="C139" s="47">
-        <v>5931.43</v>
+      <c r="B139" s="43" t="s">
+        <v>54</v>
+      </c>
+      <c r="C139" s="49">
+        <v>113.31</v>
       </c>
       <c r="D139" s="42"/>
       <c r="E139" s="42"/>
@@ -14667,14 +14667,14 @@
       <c r="H139" s="58"/>
     </row>
     <row r="140" ht="14.25" customHeight="1">
-      <c r="A140" s="46">
+      <c r="A140" s="34">
         <v>46193.0</v>
       </c>
-      <c r="B140" s="43" t="s">
-        <v>54</v>
-      </c>
-      <c r="C140" s="49">
-        <v>113.31</v>
+      <c r="B140" s="42" t="s">
+        <v>87</v>
+      </c>
+      <c r="C140" s="47">
+        <v>120.0</v>
       </c>
       <c r="D140" s="42"/>
       <c r="E140" s="42"/>
@@ -14683,13 +14683,13 @@
     </row>
     <row r="141" ht="14.25" customHeight="1">
       <c r="A141" s="34">
-        <v>46193.0</v>
+        <v>46205.0</v>
       </c>
       <c r="B141" s="42" t="s">
-        <v>87</v>
-      </c>
-      <c r="C141" s="47">
-        <v>120.0</v>
+        <v>40</v>
+      </c>
+      <c r="C141" s="49">
+        <v>930.0</v>
       </c>
       <c r="D141" s="42"/>
       <c r="E141" s="42"/>
@@ -14700,41 +14700,41 @@
       <c r="A142" s="34">
         <v>46205.0</v>
       </c>
-      <c r="B142" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="C142" s="49">
-        <v>930.0</v>
-      </c>
-      <c r="D142" s="42"/>
-      <c r="E142" s="42"/>
+      <c r="B142" s="43" t="s">
+        <v>94</v>
+      </c>
+      <c r="C142" s="47">
+        <v>400.0</v>
+      </c>
+      <c r="D142" s="35"/>
+      <c r="E142" s="35"/>
       <c r="G142" s="57"/>
       <c r="H142" s="58"/>
     </row>
     <row r="143" ht="14.25" customHeight="1">
       <c r="A143" s="34">
-        <v>46205.0</v>
+        <v>46209.0</v>
       </c>
       <c r="B143" s="43" t="s">
-        <v>94</v>
-      </c>
-      <c r="C143" s="47">
-        <v>400.0</v>
-      </c>
-      <c r="D143" s="35"/>
-      <c r="E143" s="35"/>
+        <v>60</v>
+      </c>
+      <c r="C143" s="49">
+        <v>950.0</v>
+      </c>
+      <c r="D143" s="42"/>
+      <c r="E143" s="42"/>
       <c r="G143" s="57"/>
       <c r="H143" s="58"/>
     </row>
     <row r="144" ht="14.25" customHeight="1">
-      <c r="A144" s="34">
-        <v>46209.0</v>
+      <c r="A144" s="46">
+        <v>46210.0</v>
       </c>
       <c r="B144" s="43" t="s">
-        <v>60</v>
-      </c>
-      <c r="C144" s="49">
-        <v>950.0</v>
+        <v>44</v>
+      </c>
+      <c r="C144" s="47">
+        <v>110.0</v>
       </c>
       <c r="D144" s="42"/>
       <c r="E144" s="42"/>
@@ -14745,14 +14745,14 @@
       <c r="J144" s="41"/>
     </row>
     <row r="145" ht="14.25" customHeight="1">
-      <c r="A145" s="46">
-        <v>46210.0</v>
-      </c>
-      <c r="B145" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="C145" s="47">
-        <v>110.0</v>
+      <c r="A145" s="34">
+        <v>46213.0</v>
+      </c>
+      <c r="B145" s="35" t="s">
+        <v>78</v>
+      </c>
+      <c r="C145" s="49">
+        <v>65.0</v>
       </c>
       <c r="D145" s="42"/>
       <c r="E145" s="42"/>
@@ -14764,13 +14764,13 @@
     </row>
     <row r="146" ht="14.25" customHeight="1">
       <c r="A146" s="34">
-        <v>46213.0</v>
-      </c>
-      <c r="B146" s="35" t="s">
-        <v>78</v>
+        <v>46214.0</v>
+      </c>
+      <c r="B146" s="42" t="s">
+        <v>42</v>
       </c>
       <c r="C146" s="49">
-        <v>65.0</v>
+        <v>95.12</v>
       </c>
       <c r="D146" s="42"/>
       <c r="E146" s="42"/>
@@ -14779,13 +14779,13 @@
     </row>
     <row r="147" ht="14.25" customHeight="1">
       <c r="A147" s="34">
-        <v>46214.0</v>
-      </c>
-      <c r="B147" s="42" t="s">
-        <v>42</v>
-      </c>
-      <c r="C147" s="49">
-        <v>95.12</v>
+        <v>46215.0</v>
+      </c>
+      <c r="B147" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="C147" s="47">
+        <v>981.88</v>
       </c>
       <c r="D147" s="42"/>
       <c r="E147" s="42"/>
@@ -14796,11 +14796,11 @@
       <c r="A148" s="34">
         <v>46215.0</v>
       </c>
-      <c r="B148" s="43" t="s">
-        <v>64</v>
-      </c>
-      <c r="C148" s="47">
-        <v>981.88</v>
+      <c r="B148" s="42" t="s">
+        <v>71</v>
+      </c>
+      <c r="C148" s="49">
+        <v>2831.4</v>
       </c>
       <c r="D148" s="42"/>
       <c r="E148" s="42"/>
@@ -14811,11 +14811,11 @@
       <c r="A149" s="34">
         <v>46215.0</v>
       </c>
-      <c r="B149" s="42" t="s">
-        <v>71</v>
+      <c r="B149" s="43" t="s">
+        <v>56</v>
       </c>
       <c r="C149" s="49">
-        <v>2831.4</v>
+        <v>50.0</v>
       </c>
       <c r="D149" s="42"/>
       <c r="E149" s="42"/>
@@ -14823,14 +14823,14 @@
       <c r="H149" s="58"/>
     </row>
     <row r="150" ht="14.25" customHeight="1">
-      <c r="A150" s="34">
-        <v>46215.0</v>
+      <c r="A150" s="46">
+        <v>46218.0</v>
       </c>
       <c r="B150" s="43" t="s">
-        <v>56</v>
-      </c>
-      <c r="C150" s="49">
-        <v>50.0</v>
+        <v>91</v>
+      </c>
+      <c r="C150" s="47">
+        <v>60.0</v>
       </c>
       <c r="D150" s="42"/>
       <c r="E150" s="42"/>
@@ -14838,14 +14838,14 @@
       <c r="H150" s="58"/>
     </row>
     <row r="151" ht="14.25" customHeight="1">
-      <c r="A151" s="46">
+      <c r="A151" s="34">
         <v>46218.0</v>
       </c>
       <c r="B151" s="43" t="s">
-        <v>91</v>
-      </c>
-      <c r="C151" s="47">
-        <v>60.0</v>
+        <v>62</v>
+      </c>
+      <c r="C151" s="49">
+        <v>132.4</v>
       </c>
       <c r="D151" s="42"/>
       <c r="E151" s="42"/>
@@ -14853,14 +14853,14 @@
       <c r="H151" s="58"/>
     </row>
     <row r="152" ht="14.25" customHeight="1">
-      <c r="A152" s="34">
+      <c r="A152" s="46">
         <v>46218.0</v>
       </c>
       <c r="B152" s="43" t="s">
-        <v>62</v>
-      </c>
-      <c r="C152" s="49">
-        <v>132.4</v>
+        <v>103</v>
+      </c>
+      <c r="C152" s="47">
+        <v>50.0</v>
       </c>
       <c r="D152" s="42"/>
       <c r="E152" s="42"/>
@@ -14869,13 +14869,13 @@
     </row>
     <row r="153" ht="14.25" customHeight="1">
       <c r="A153" s="46">
-        <v>46218.0</v>
-      </c>
-      <c r="B153" s="43" t="s">
-        <v>103</v>
-      </c>
-      <c r="C153" s="47">
-        <v>50.0</v>
+        <v>46222.0</v>
+      </c>
+      <c r="B153" s="42" t="s">
+        <v>66</v>
+      </c>
+      <c r="C153" s="49">
+        <v>530.0</v>
       </c>
       <c r="D153" s="42"/>
       <c r="E153" s="42"/>

</xml_diff>